<commit_message>
docs: update the consolidated defect register and roadmap backlog spreadsheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/product-road-map/Refined-Road-Map/HireBuddha-Roadmap-Backlog.xlsx
+++ b/docs/product-road-map/Refined-Road-Map/HireBuddha-Roadmap-Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\Development\hire-buddha-app\docs\product-road-map\Refined-Road-Map\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3231628-E521-477A-884B-18C3D21271D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5551295-4658-470E-B566-76C1FCB87FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,6 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'HireBuddha Roadmap Backlog'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3376" uniqueCount="1244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3409" uniqueCount="1277">
   <si>
     <t>HireBuddha — Refined product roadmap: all epics, features and user stories</t>
   </si>
@@ -3989,6 +3988,694 @@
   </si>
   <si>
     <t>Description</t>
+  </si>
+  <si>
+    <t>Functional requirements — Skills and controlled capabilities
+Purpose: reusable business capabilities must be authored as Skills, with controlled tools enforcing their effects. The Skill tier and some dynamic-tool code exist, but the version and asset model is new. Depends on E01–E05 and E12's sandbox controls. Decision D04 confirms Skills as the main authoring unit. References: SK throughout, GTM §6, FEAS N-6/N-7, and the TL, EP and MI defects.
+A Skill author must be able to create a reusable capability with instructions, input and output contracts, scripts and assets.
+Database-backed drafts must describe their purpose, discovery information, permitted primitives, governance and runtime reference.
+Published versions must be immutable, with working comparison, testing, publication and rollback. Each execution must pin and record its chosen version.
+A workforce designer must be able to reuse a Skill without adding unnecessary agent reasoning loops.
+Eligible Skills must first expose brief metadata, with full instructions loaded when selected. Selection must respect access and suitability for the task.
+Direct invocation and optional Action wrappers must both work. Multiple consumers must be able to share one version without indiscriminately copying ownership or memory.
+A tenant administrator must be able to run authored scripts without exposing credentials or the host environment.
+Approved runtime images must supply dependencies. Assets must be verified by hash and isolated by tenant, version and run where needed.
+Authored code must not install packages at runtime or fall back to host execution. Resource, network and file limits must be enforced, and external credentials must remain behind controlled tools.
+An operator must be able to enable a capability once and use it across workers and restarts.
+Registry entries must resolve to executable implementations, and workers must reload the correct version of each tenant capability.
+Discovery and execution must both check tenant, enabled status and permissions. Disabling a capability must take effect everywhere, and unknown definitions must not execute.
+An operator must be able to generate documents reproducibly through the reference Skill family.
+Deterministic DOCX, PPTX, PDF and spreadsheet boilerplate must become stored scripts and assets, while prompts retain work requiring judgment.
+Outputs must be registered artifacts. Tests must compare quality, token use, latency and cost with the existing path, and attribute usage to the Skill version and sandbox.
+A capability owner must be able to consolidate social and integration wrappers without losing controls.
+Selected operations must be piloted through authenticated controlled primitives and platform Skills, retaining operation permissions, consent, idempotency and budgets.
+Migration must compare task quality and cost, support rollback, and retire old paths only after a verified cutover.</t>
+  </si>
+  <si>
+    <t>Functional requirements — connections and system-of-record sync
+Purpose: connecting an external system must produce usable, recoverable capabilities with clear data ownership. Some adapters exist, while MCP transport and complete synchronization are new. Depends on E01, E03 and E08, and on E06/E07 for record synchronization. Under D02, hybrid mastering and HubSpot as the first reference connector remain proposals requiring confirmation. References: GTM §§4 and 7, FEAS N-6, RT §21, and the TL defects.
+An administrator must be able to connect, test, rotate credentials for, and revoke an external service.
+Setup must show supported operations and scopes, the connected account, test results, health and limits.
+Credentials must be encrypted and excluded from model prompts. Expired tokens must produce an actionable reconnect state.
+Revocation must disable dependent effects and identify the workflows affected.
+An administrator must be able to attach an approved MCP server and use its permitted capabilities.
+The chosen transport must work end to end, and saved configuration must reconnect on every worker.
+Discovering a tool must not itself grant permission to execute it. Server metadata must be treated as untrusted, with explicit operation policies and limits applied independently.
+Timeouts, outages and revocations must have visible outcomes.
+A CRM owner must be able to declare the authoritative system for each object and trust the local mirror.
+External identifiers, field mappings and freshness must be visible. Writes to externally mastered records must wait for confirmed write-back.
+Conflicts must preserve the losing change for review. Retries and webhook replays must neither duplicate records nor cause changes to oscillate between systems.
+An owner must be able to move an object deliberately between local and external mastering.
+Migration must preview affected records, relationships, consent and conflicts, preserve a recovery snapshot, backfill mappings, reconcile counts and obtain required approval.
+Partial failures must support resumption or rollback. A connector outage must never silently change the authoritative system.
+A business user must be able to synchronize the knowledge and collaboration sources their workflow needs.
+Drive, SharePoint, Notion, Slack and Teams must be prioritized according to the chosen pilot. The Cortex acquisition path must also support the approved OneDrive scope described in E38.
+Synchronization must respect source permissions, changed and deleted documents, and progress cursors. Review cards must use the same authenticated approval service as other interfaces.
+Every advertised integration must pass a representative end-to-end use case.
+An administrator must be able to distinguish available, preview, unavailable and planned capabilities in the integration catalog.
+The catalog must cover calendar, email, CRM, analytics, enrichment, e-signature, payments, bank feeds, tax, HRIS, inventory and helpdesk families.
+Enabling an integration must require evidence that connection, metering, policy enforcement and recovery work.</t>
+  </si>
+  <si>
+    <t>Functional requirements — Pragya and business onboarding
+Purpose: an owner must be able to turn business goals into a reviewable operating setup and supervise it through Pragya. This is a new experience built on partial entity-builder and Board capabilities. Depends on E01, E03, E05 and E08, and E06/E09 for connected operations. Decisions D26 and D30 establish Pragya as the single, voice-first human workspace and require collaborative solution design. References: RF §§4–5, GTM §11, RT §11, and the MI defects.
+A new owner must be able to establish business context without answering questions the product can already resolve.
+Pragya must research supplied and public sources, show its assumptions, ingest approved internal sources and revise conclusions with provenance.
+It must ask only unresolved questions and must never save a speculative business fact as verified. Discovery must support pausing and resuming.
+An owner must be able to agree workflows, intended outcomes and boundaries before deployment.
+Planning must capture business problems, owners, priorities, KPIs, budgets, data and mastering choices, permitted channels and review rules.
+The proposal must identify required Skills, integrations and missing capabilities, with changes available for review. A Solo Pack or fixed agent roster must not be mandatory.
+A designer must be able to request a capability and receive an editable, tested candidate.
+The builder must look for reusable capabilities before creating new ones and must be able to revise failed candidates.
+Tests must include independent known cases, failures and permission boundaries. Skipped tests and tests stopped by an exhausted budget must not count as passes.
+Generated work must remain a draft until an authorized person promotes it.
+An owner must be able to preview a business workflow realistically before activating it.
+The preview must show representative inputs and outputs, approval points, records affected, dependencies and estimated costs without causing live effects.
+Missing credentials or policies must block activation. Deployment must use pinned versions and the chosen autonomy policy.
+An owner must be able to ask what happened, what needs attention and what it cost.
+Pragya must answer from actual records and runs, link the evidence, distinguish observed results from estimates, and show pending reviews, failures and business outcomes.
+Requested changes must pass the same permissions and approval controls as direct UI actions.
+An owner must be able to continue through voice, text or a verified collaboration channel, with channels introduced only when their adapters have demonstrated readiness.
+Authorized identity and permitted context must survive handoff. Private reports must not reach external counterparties, and unverified or sensitive requests must receive the required verification.
+A failed channel must offer a valid fallback. Text, directly editable views and immediate stop controls must remain available within the Pragya workspace.</t>
+  </si>
+  <si>
+    <t>Functional requirements — Karuna and communication channels
+Purpose: customer-facing interactions must share conduct rules, identity, history and escalation behavior. Voice, email and messaging paths exist with major gaps. Depends on E01–E05, E07–E09 and E06's consent and activity records. D03 requires an approved workflow policy for routine effects, exception and mandatory-checkpoint review, and an explicit session policy for live voice. D06 requires funded safe closure without intentional debt, and D28 requires complete Exotel integration. References: GTM §§3, 8 and 11, FEAS §§2–4, BP §2.3, and the VT, GW and TL defects.
+An owner must be able to enforce contact permission and conduct before every external action.
+Email, calling, messaging, social, browser and connector paths must check consent and purpose, suppression, recipient or account ownership, time windows, disclosure policy and required human review immediately before execution.
+Policy failure must block the action, and prompts must not override it.
+A customer must be able to set contact preferences, stop contact and request a human.
+Opt-out must promptly update shared suppression and stop queued and future prohibited contact. Verified preferences must apply across linked channels.
+A human request must create an owned handoff. If nobody is available, the customer must receive an honest callback or response expectation.
+An operator must be able to run inbound and outbound voice under an approved session policy.
+Carrier routing, recording and disclosure choices, interruption, tool calls, costs, disposition and activity linkage must work end to end.
+Consent and funds must be checked before dialing, every tool effect must use platform controls, and safe closure must be funded in advance. Low credit or an outage must not cause intentional debt.
+An operator must be able to handle email, messaging and web conversations through a coherent inbox showing threads, participant identity, attachments, delivery state and assignment.
+Reconnects and retries must not duplicate sends. Uncertain delivery must not be reported as successful.
+Handoffs must carry permitted history without exposing private operator conversations.
+A customer must receive appropriate communication in a supported language, following brand tone and accessibility rules.
+Language detection and translation must disclose uncertainty and preserve material meaning. Unsupported languages must route to help.
+Persona settings must affect delivery without promising a guaranteed emotional response from a numeric setting.
+An operator must be able to recover from a channel outage while respecting the fallback channel's consent and customer preferences.
+Queued work must retain ordering and stop rules. Callback promises must create owned tasks.
+Real-time streams must be authenticated and resumable where possible. Failed sessions must preserve trustworthy cost and outcome records.
+An owner must be able to connect Exotel for approved calling use cases with tenant-scoped credentials, verified account and number ownership, signed webhooks, regional settings, and recording and disclosure policy.
+Connection health and capability limits must be visible. Unsupported use cases comparable to Smartflo must fail clearly.
+Exotel inbound and outbound setup, answer, busy, no-answer, failure, transfer, hangup and human handoff must map to durable call and activity records.
+Consent, suppression, schedules and funds must be rechecked immediately before dialing.
+Signed callbacks must be reconciled idempotently. Delayed, duplicate and out-of-order events must not move a call back to an earlier state.
+Recording references, consent, retention and access must be stored in the tenant data plane, with unknown outcomes surfaced for review.
+Timeouts, rate limits, provider outages and missing webhooks must trigger bounded retry and reconciliation without blind redial or duplicate business effects.
+Metered costs and closure reserves must settle accurately, and fallback and emergency-stop behavior must be tested.</t>
+  </si>
+  <si>
+    <t>Functional requirements — operational readiness and service continuity
+Purpose: the product must be demonstrable, releasable, recoverable and supportable with evidence. The application exists with substantial release and operational defects. This work is cross-cutting and must be delivered alongside the capabilities it protects. D25 defines tenant-data placement, and D33 requires defects to be revalidated rather than assumed closed by replacement. References: DR, the FE, TS, IN, SA, DM and API registers, and GTM §4.2.
+A developer must be able to start a fresh local checkout without production domains or credentials.
+The supported environment, dependencies, migrations and fixtures must be documented. Local URLs must be explicit, and missing configuration must never default to production.
+Mock and offline tests must be distinguishable from live-provider tests. Public callback setup must be separate from basic local operation.
+A release owner must be able to establish that required checks actually ran.
+Continuous integration must trigger for active backend and frontend paths and report executed counts for required unit, integration, UI and regression tests.
+Missing infrastructure must fail required checks. Security and tenant isolation, approvals, money and replay scenarios must exercise real dispatch paths, and documentation must identify unverified services accurately.
+An operator must receive useful error, loading, empty and permission states, reconnect guidance and actionable request identifiers.
+Metrics must expose policy failures, queue age, approvals, cost mismatches, connector health and run outcomes. Log access must be scoped and secrets redacted.
+A tenant owner must be able to recover or export the complete supported business state.
+Encrypted automated backups must begin before operational writes. Restore drills must include record versions and relationships, knowledge, memory, configuration, relevant history and ledgers, and artifact manifests.
+Exports must be usable and tenant-scoped, exclude raw credentials and identify missing external data. Recovery and acceptable data-loss targets must be agreed and measured.
+A service owner must be able to operate tenant databases independently of code execution.
+Database sleep and startup, connection pools, durable volumes, upgrades, capacity and backups must have explicit lifecycle controls.
+Work must park when its tenant database is waking or unavailable. Readiness must be monitored per tenant, and persistent storage must not depend on local scratch directories.
+A product owner must be able to decide whether a release is supportable.
+Every enabled capability must have a supported-version record, an owner, a rollback procedure, an operating runbook and acceptance evidence.
+Blockers and unresolved defects must be explicit. Unsupported tools must be inaccessible, and superseded runtime paths must be removed after verified migration and the defined rollback-retention period.
+Before work starts in an area, its numbered defect register must be checked against the current code and runtime path.
+Each item must be classified as applicable-repair, replaced-path, not-reproducible, deferred or accepted-risk, with evidence, an owner and a date. Duplicate identifiers must remain cross-referenced without double counting.
+Applicable T0 and T1 defects must become release-blocking stories or tests in the responsible epic.
+Fixes must be verified through API, worker, tool, UI and external-provider paths where relevant. Feature flags and seed data must not count as proof, and missing infrastructure must not allow tests to pass by silently skipping.
+Closing a defect must link the change, regression evidence and current behavior. Replacing a component must not automatically close its defects.
+Deferrals must record the reason, mitigation and review date. Unresolved defects must remain visible in release readiness and must not be relabelled as completed features.</t>
+  </si>
+  <si>
+    <t>Functional requirements — market intelligence and targeting
+Purpose: marketing and sales teams must build a defensible understanding of markets, accounts and audiences. Research and artifact tools exist, while durable business intelligence is new. The primary operators are marketing and revenue operations. Depends on E01–E05 and E08, with E06 for records, E07 for monitoring, E09 for connected sources and E11 for any external communication. References: GTM §§6 and 9, and FEAS §2.
+A marketer must be able to produce a cited company, market or competitor brief through a reusable Skill.
+Findings must identify their source and observation date, distinguish claims from inference, and flag inaccessible or conflicting evidence.
+The brief must be downloadable without being published externally.
+A marketer must be able to monitor news, pricing and feature changes, hiring, funding, reviews and category developments without repeated alerts for the same observation.
+Scheduled research must compare new observations with prior records. Deduplication must retain provenance, and meaningful changes must create owned Business Signals.
+Unknown data must not become a fabricated trend.
+A revenue owner must be able to define and revise an ideal customer profile with explainable scoring.
+Rules, weights and disqualifiers must be versioned. Scores must show supporting evidence and missing fields.
+A revised definition must support rescoring a preview cohort before activation. Enrichment must obey restrictions on protected and sensitive data.
+A seller must be able to build target-account and buying-group lists from permitted evidence.
+Account and contact enrichment must record source, freshness and confidence. Identity deduplication must use E06, and saved segment criteria must reproduce the same selection logic.
+Finding contact details must never imply permission to contact. A vendor enrichment service must be replaceable behind the same Skill contract.
+A seller must be able to prepare account briefs, competitive battlecards and evidence for responding to objections.
+Outputs must use the current approved messaging library and cite sources, mark unsupported comparisons, and restrict sensitive customer evidence to permitted users.
+The brief version must link to the relevant account or deal.
+An owner must be able to turn an insight into a proposed campaign, account task, risk or product idea and later assess its value.
+The receiving owner must accept or reject the proposal with a reason. Resulting work and outcomes must link to the original insight.
+Read-only research must not silently trigger an external send.</t>
+  </si>
+  <si>
+    <t>Functional requirements — content and demand generation
+Purpose: a brand owner must be able to move from evidence-backed briefs to reviewed assets, publication and measured learning. Content, media and document tools exist, while brand records, editorial workflow and governed distribution are new. Depends on E01–E05, E08, E06 for editorial records, E07 for scheduling, E09/E11 for publishing, and E04-S06 for paid commitments. D03 governs approved workflow policy and exceptions. References: GTM §§6 and 8–11, SK, and FEAS N-2/N-3/N-9.
+A brand owner must be able to maintain approved positioning, proof points, tone and prohibited claims in a versioned, permissioned Messaging Library.
+Content Skills must retrieve approved material. Brand and factual reviews must identify offending passages and supporting evidence, and missing evidence must produce an explicit gap.
+A content operator must be able to create and repurpose articles, landing-page copy, case studies, newsletters, social posts, one-pagers, decks, video scripts and advertising variants for a defined audience and channel.
+Derived assets must retain claim provenance. Documents and media must have previews and linked artifacts, and reusable scripts must avoid repeatedly generating boilerplate.
+An editor must be able to manage a content calendar and review the exact asset intended for publication.
+Brief, draft, review, approved, scheduled, published and failed states must be visible. Reviewer edits must retain version history, and subsequent asset changes must invalidate approval.
+The schedule preview must show channel, account and timezone. Rejected work must return to an assigned owner.
+A marketer must be able to publish approved content to validated channels and verify completion.
+Current account permissions, policy and idempotency must be checked before publication. Provider acceptance must be distinguished from actual publication.
+The final URL, status and metrics must link to the asset. Partial failure across channels must retry only unresolved effects that remain eligible.
+A marketer must be able to run event, community, review and nurture programs with governed follow-up.
+Registrations, invitations, attendance and no-shows, replies, reminders and follow-up must become records or activities and obey consent and stop rules.
+Public-relations statements must receive named approval. Complaints and sensitive community responses must route to an accountable human.
+A paid-marketing owner must be able to plan and optimize advertising within explicit spending limits.
+The preview must show campaign, audience, creative and external advertising budget separately from platform costs.
+Spend-changing actions must follow configured approval bands. Pacing must use reconciled provider actuals and commitments, and missing spending data must stop increases.
+Search optimization, conversion optimization and advertising experiments must distinguish recommendations from changes actually applied.</t>
+  </si>
+  <si>
+    <t>Functional requirements — inbound qualification and booking
+Purpose: an inquiry must become an identified, owned opportunity or a correctly routed service request. Voice and gateway components exist, but reliable capture, qualification and booking are new workflows. Depends on E01–E05, E08, E06/E07/E09/E11 and D03's approved workflow and voice-session policy. References: GTM-P4, FEAS N-5, and the GW and VT defects.
+A sales operator must be able to capture inquiries from supported forms, web chat, email, messaging and phone channels.
+Capture must persist the source, time, contact permission and supplied details. Signatures and rate limits must protect intake.
+Repeated submissions must not create duplicate work. Routing must never choose an arbitrary Action or Skill, and unanswered or unroutable inquiries must enter an owned queue.
+A seller must be able to see a new inquiry alongside earlier interactions.
+Identity matching must be explainable and reversible, and account, contact and activity records must retain attribution.
+Existing-customer and support requests must route appropriately. Anonymous or uncertain identities must remain separate until resolved.
+A sales manager must be able to qualify and assign inquiries using explicit business rules.
+Versioned fit and intent scores must show evidence. Assignment must follow capacity, territory and availability rules, with a fallback owner.
+Inactivity must trigger the configured service-level escalation. Model uncertainty must not invent eligibility or a qualification answer.
+A prospect must receive a relevant response using approved product and price facts and permitted history, with an appropriate route to a human.
+Responses must follow the approved workflow or session policy and required exception review. Response-time reporting must distinguish human-review waiting from AI processing.
+Human-escalation requests and opt-outs must be honored.
+A prospect must be able to book a valid meeting in their timezone.
+Availability must be checked before booking, with working hours, buffers, round-robin assignment and attendee timezones applied.
+A last-minute conflict must produce alternatives. Only one provider-confirmed event must be created and linked to the opportunity or activity.
+A prospect or representative must be able to reschedule or cancel and receive appropriate reminders or no-show follow-up.
+Changes must update the same meeting, cancel obsolete reminders and preserve history. Provider failures must be visible.
+Follow-up must use current consent and reply state, and attendance or outcome must close the original booking task.</t>
+  </si>
+  <si>
+    <t>Functional requirements — outbound sequences and deliverability
+Purpose: approved outreach must happen at the right time and stop when required. Single-message SMTP and dialer infrastructure exist, while sequences and deliverability controls are new. Depends on the shared E01–E05/E08 foundations, E06/E07/E09/E11, durable approvals and budget controls. A live outbound pilot must wait for those prerequisites. D03 permits routine effects within an approved workflow policy and requires review of exceptions and mandatory checkpoints. References: GTM §§3, 5 and 8–11, and FEAS §3/N-3/N-9.
+An outbound operator must be able to validate a sender and its limits before launch.
+Provider connection, domain authentication and readiness, mailbox identity, daily caps and volume ramp must be visible. Missing setup must block launch.
+Bounce and complaint thresholds must pause affected sending. Rotating mailboxes must not bypass account or domain limits.
+A contact must be able to withdraw permission and have the change enforced immediately.
+Consent must be specific to channel and purpose and retain source, time and evidence. Unsubscribe, complaint, hard-bounce and do-not-call events must update shared suppression.
+Imported lists must not silently clear suppression. Queued steps must check eligibility again immediately before sending or dialing.
+An operator must be able to design, preview and approve a sequence before enrolling contacts.
+Versioned steps must define channel, delay, conditions, template, sending window and exit rules. Previews must show representative recipients, costs and permissions.
+Invalid schedules, loops and missing permissions must fail validation. Active enrollments must retain their selected version until explicitly migrated.
+An operator must be able to trust sequence timing and effects through retries and restarts.
+Deterministic states must determine step eligibility. Each effect must use a stable idempotency key, and leases for each recipient and enrollment must prevent concurrent sends.
+Caps and timezones must apply. Pause, cancellation and uncertain provider outcomes must survive restarts without duplicate contact.
+A seller must be able to take over when a prospect replies or books.
+Replies must link to the correct contact and thread. Replies, bookings and opt-outs must stop or alter enrollment under explicit rules, while ambiguous replies must go to review.
+The next effect must recheck state immediately before dispatch so a recent reply cannot be missed. Handoffs must include qualified context.
+A marketing owner must be able to assess results by cohort and sequence version, including delivery, replies, meetings, failures and suppression.
+Privacy-sensitive open and click tracking must be optional under policy and labelled approximate. Platform cost must be separate from delivery and advertising spend.
+Direct-message and connection automation must remain unavailable unless an approved, supported provider capability exists.</t>
+  </si>
+  <si>
+    <t>Functional requirements — deal desk and sales execution
+Purpose: sellers must be able to prepare, qualify, quote and hand off deals using shared evidence. Research and document generation are partly available, while the deal workflow is new. Depends on E06/E09, E05 for grounded answers, E03/E11 for controlled approvals and sends, and E26 for signed contracts, alongside the shared execution, spending and Skill foundations. References: GTM-P6 and GTM §9, FEAS N-2, and BP's sales inventory.
+A seller must be able to prepare a meeting brief and demo plan from verified account context.
+The brief must show stakeholders, interaction history, current needs, open questions and sources. Missing or stale CRM data must be labelled, and interaction history must not be invented.
+A reviewable artifact must be possible from approved uploads before live CRM synchronization is available.
+A seller must be able to turn an authorized recording or notes into confirmed actions and qualification evidence.
+Transcripts and notes must retain provenance and recording permissions. MEDDIC- or BANT-style fields must show evidence and unknowns.
+CRM edits must be proposed as a visible difference from current data. Confirmed actions must have owners and dates, and ingestion of external meetings must remain distinguishable from transcription of platform calls.
+A deal owner must be able to create an accurate quote or proposal within approved terms.
+The Product/Service catalog and Quote and line-item records must support quantity, currency, taxes, validity and versioning. Arithmetic must be deterministic.
+Nonstandard terms and discounts must receive required approval. Approved artifacts must link to the opportunity, and price changes must invalidate affected approvals.
+A presales specialist must be able to draft RFP and security-questionnaire responses from current, accessible, approved evidence.
+Answers must cite sources, assign gaps to experts and respect confidentiality. Claims and certifications must not be invented.
+The final response and attachments must be reviewed before dispatch.
+A manager must be able to inspect deal risks, record quality and forecast changes.
+Missing fields, stale activity, inconsistent stages, competitor and champion signals, and changes in close date must be explainable.
+Updates must follow system-of-record rules. Win and loss reasons must retain evidence, and predictions must remain distinct from confirmed bookings.
+A delivery or customer-success owner must receive an accepted closed-won handoff exactly once.
+Required approvals, signatures and commercial conditions must be verified before accepted scope, obligations, quote and contacts create linked order or onboarding work.
+The recipient must acknowledge ownership. Duplicate close events must not duplicate downstream work, and reopening or cancellation must propagate explicitly.</t>
+  </si>
+  <si>
+    <t>Functional requirements — revenue operations and reporting
+Purpose: owners must be able to trace revenue metrics to business records, interactions and costs. Platform usage reporting exists, while business reporting is new. Depends on E06, the relevant channel, CRM and payment data, and E04's cost ledger, with shared controls and Skills. References: GTM-P2 and GTM §§9–11, and the FEAS §2 correction. A generated research report is not evidence that pipeline reporting already works.
+A revenue owner must be able to inspect funnel, pipeline and conversion by cohort.
+Reports must show lifecycle and stage definitions, period, timezone, currency, deduplication rules and exclusions, with drill-down to records and activities.
+Incomplete or stale synchronization must be visible. Unavailable source data must appear as unknown, never as zero or invented revenue.
+A manager must be able to inspect forecasts and outcomes with explicit assumptions.
+Committed, best-case and forecast figures must be distinguished from won and paid results. Probability versions and missing data must be disclosed and evidence linked.
+Weekly briefs must show risks, required decisions and changed assumptions.
+A marketer must be able to compare channels using a consistent attribution model whose limits are stated.
+First-touch, last-touch and self-reported sources must be available. Conversion windows and identity gaps must be explicit, and multi-touch attribution must not be presented as proof of causation.
+Campaign, content and sequence lineage must survive record merges and CRM synchronization.
+An owner must be able to inspect cost per qualified opportunity, meeting and sale.
+Platform, provider and campaign costs must reconcile to their ledgers and the relevant outcome cohort.
+Cancelled, duplicate and failed activities must be treated consistently. Missing external spend must be disclosed, and margin and return-on-investment calculations must show assumptions.
+An owner must be able to see what the AI workforce did and what needs attention through an activity feed filtered by business object, workflow and outcome.
+The feed must link runs, costs, approvals and artifacts, including failures, skipped actions and waiting work.
+The business result must be understandable without reading raw internal traces.
+A revenue-operations owner must be able to turn performance findings into controlled improvement proposals.
+Alerts must use configured thresholds and data freshness. Proposals must identify affected Skills or rules and their evidence, while human edits and rejections must feed evaluation.
+A recommendation must not silently change pricing, outreach or policy.</t>
+  </si>
+  <si>
+    <t>Functional requirements — customer care, retention, and expansion
+Purpose: customers must receive continuous, accountable help from onboarding through renewal. Channel and knowledge-base components exist, while customer operations are new. Depends on E05/E06/E07/E09/E11/E18 and the shared platform controls. This is an H4 module, supporting local records and declared external masters. It adds Ticket, Customer Onboarding Plan, Service Entitlement, Health Snapshot and Renewal records, reusing Account, Contact, Activity and Opportunity. References: GTM §9's lifecycle signals and BP's support, retention and education inventory.
+A customer must be able to report a problem across supported channels and receive an accountable response.
+Intake must create or deduplicate a ticket, determine entitlement and priority, assign an owner and response deadline, and link related conversations.
+Urgent and security cases must route to the appropriate incident owner. Closure must record a resolution or an explicit unresolved state.
+A support operator must be able to resolve known issues from approved evidence and escalate the rest.
+Suggested answers must cite current knowledge and product context. Diagnostic tools must use scoped permissions.
+Low confidence, failed remediation and requests for a human must trigger handoff with history. Customer responses must follow communication policy, and feedback may propose a knowledge-base update for review.
+A customer-success owner must be able to turn the accepted sales promise into an onboarding plan.
+The plan must include customer goals, commitments, tasks, owners, dates and acceptance conditions. Completion must be supported by evidence, blocked tasks must escalate, and scope changes must require an explicit decision.
+Customer appointments must reuse the existing booking capability.
+A customer must be able to obtain relevant training and approved self-service material.
+Guides and tutorials must be versioned and linked to the applicable product and entitlement. Completion and unresolved questions must be recorded.
+Repeated questions must be able to propose content improvements. Inaccessible or obsolete material must not be presented as current guidance.
+An account owner must be able to identify customers at risk or ready for expansion and act on the evidence.
+Health must combine declared usage, support and payment inputs with freshness and explainable weights. Risks must create assigned interventions, and renewal dates must trigger governed tasks.
+New commercial terms must use quote and contract approval rather than silent account changes.
+An account owner must be able to prepare quarterly business reviews, feedback surveys and advocacy requests.
+Review metrics must link to records, and surveys and review requests must obey consent and contact policy.
+Complaints must route to service recovery. Case studies and public references must have customer permission, and participation must be measured separately from satisfaction.</t>
+  </si>
+  <si>
+    <t>Functional requirements — orders, delivery, and fulfillment
+Purpose: an accepted commercial promise must become a tracked, delivered and accepted product or service. This is a new H4 business module using shared records, events, Skills, integration ownership and platform controls. Depends on E06/E07/E17/E26, E22 for purchased inputs and E21 for billing. It adds Order/Line, Project, Task, Milestone, Deliverable, Acceptance, Shipment and Return records and reuses the Product/Service catalog. References: GTM's closed-won handoff and BP's delivery inventory.
+A delivery manager must be able to plan accepted work against capacity and dependencies.
+Approved scope must create one linked order or project. Tasks must identify owners, required resources, dependencies and deadlines, and overcommitment must be visible.
+Scope changes must preserve the original commitment and obtain required approval.
+A customer or authorized reviewer must be able to inspect a deliverable, accept it or request rework.
+Completion must require the specified evidence and reviewer authority. Quality checks and proof of work must remain linked to the deliverable.
+Partial acceptance and rework must remain visible. An accepted milestone must emit only one eligible billing or handoff event.
+An operations owner must be able to fulfill stocked goods or provision a service without promising unavailable capacity.
+Inventory or resource availability must be checked and reserved before confirmation. Shipment and provisioning status must come from actual execution or provider evidence.
+Failures must create owned exceptions. Detailed production and bill-of-materials planning must remain an optional, separately scoped capability.
+A service operator must be able to manage delays, returns and corrective action.
+Service-level risks must alert the accountable owner, and customer communications must receive required review.
+Returns must track eligibility, receipt, inspection and disposition. Refunds must use the authorized finance workflow.
+Order, project and inventory state must reconcile after cancellation or retry.</t>
+  </si>
+  <si>
+    <t>Functional requirements — invoicing and collections
+Purpose: accepted commercial obligations must become correct invoices, receipts and reconciled balances. This is a new H4 business-finance module, separate from HireBuddha's platform billing. Depends on E04's external-commitment controls, E06/E07/E09/E11/E17, E23 for accounting and the shared approval and execution services. It adds Invoice/Line, Receivable, Receipt, Credit Note and Collection Case records and reuses Order, Contract and Payment. References: BP's receivables inventory, RT's HBS concept and the GTM payment-attribution extension.
+A finance operator must be able to issue a reviewed invoice from accepted terms or delivered milestones.
+Amounts, taxes, currency, numbering, due date and billing party must be validated. Draft, issued, void and credited states must be explicit.
+Issued history must remain immutable and be corrected through adjustments. Repeated milestone events must not produce duplicate invoices.
+A finance operator must be able to record and allocate payments accurately.
+Provider callbacks and imports must have their source verified and be deduplicated. Partial payments, overpayments, underpayments and fees must be explicit.
+Receipt allocations must reconcile to outstanding invoice amounts. Failed or reversed settlement must reopen the appropriate balance while retaining history.
+An accounts-receivable owner must be able to follow up on overdue balances with the correct context and contact limits.
+Deterministic reminders must use the current outstanding balance, agreed time windows and contact policy.
+Disputes, confirmed payment and manual holds must stop inappropriate reminders. Collection actions and promises to pay must have recorded owners and dates.
+A finance reviewer must be able to resolve a dispute or approve a credit, refund or write-off.
+The review must include contract, delivery and support evidence and show financial impact. Required independent and authorized approval must apply.
+The adjustment must update receivables and accounting exactly once. The customer must receive only the approved outcome, and the complete case must remain auditable.</t>
+  </si>
+  <si>
+    <t>Functional requirements — procurement and payables
+Purpose: goods and services must be purchased, and suppliers paid, under controlled authority. This is a new H4 module using the shared platform services and declared system-of-record ownership. Depends on E03/E04/E06/E07/E09/E23/E26. It adds Vendor Profile, Requisition, Purchase Order, Goods/Service Receipt, Supplier Bill, Payment Instruction and Verification Result records. References: BP's procurement, vendor and payables inventory, and RT's ownership and separation-of-duties requirements.
+A procurement owner must be able to assess suppliers and activate an approved vendor.
+Vendor identity, risk, insurance and compliance documents, and verification freshness must be recorded. Adverse findings must escalate.
+Bank-detail changes must receive independent verification. The person who creates a vendor must not authorize its payment.
+A requester must be able to obtain an approved purchase for a documented business need.
+The requisition must compare available suppliers, terms and budget. Approval must create a versioned purchase order.
+Changes and cancellations must update commitments, and the requester must be able to see delivery or service acceptance and any exceptions.
+An accounts-payable operator must be able to match a bill to authorized purchasing and receipt evidence.
+Duplicate-invoice checks and checks of amounts, quantities, taxes and purchase-order or receipt tolerances must be deterministic.
+Unmatched differences must create an owned exception. Matching a bill must not itself authorize payment.
+An authorized payer must be able to execute a reviewed payout and know the settlement outcome.
+Beneficiary, bank-detail version, amount, currency, due date, authority and funds must be rechecked before payment.
+Maker/checker separation and dual-approval rules must apply. Stable idempotency and provider reconciliation must prevent duplicate payouts.
+Pending, failed and reversed transactions must remain distinguishable from paid transactions.</t>
+  </si>
+  <si>
+    <t>Functional requirements — accounting and financial close
+Purpose: tenants must be able to maintain consistent business books with traceable evidence. This is a new H4 module; platform usage logs do not constitute business accounts. Depends on E06/E09, transactional feeds from E21/E22, E03 review and the shared platform services. It adds Chart of Accounts, Journal/Entry/Line, Accounting Period, Bank Statement/Line, Reconciliation, Expense Claim and Tax Code records. References: BP's accounting, expenses and tax inventory, and RT's HBS concept. Supported local scope and externally mastered accounting must be declared explicitly.
+An accountant must be able to post balanced, evidence-backed transactions and correct them visibly.
+Deterministic double-entry checks must prevent imbalanced entries. Currency, posting date and account must be validated.
+Posted entries must be immutable, with corrections recorded as reversals or adjustments. Open and closed accounting periods must be enforced.
+Source documents and approved business events must link to the entries they support.
+A bookkeeper must be able to reconcile bank and payment records and employee expenses.
+Imports must be deduplicated and retain their source. Suggested matches must show evidence and confidence, and approved matches must be distinguished from unmatched exceptions.
+Expense claims must include receipts, policy checks and review. Adjustments must not bypass accounting controls.
+A finance owner must be able to close a period and produce reconciled management accounts.
+The close checklist must cover unresolved matches, receivables, payables and required adjustments. The trial balance and supported statements must reconcile to journal entries.
+Reopening a period must require authority. Missing inputs must prevent a claim that the close is complete without exceptions.
+A domain reviewer must be able to configure supported taxes and prepare required financial reports.
+Tax and jurisdiction rules must be versioned with sources and effective dates. Arithmetic must follow deterministic rules or approved providers.
+Unsupported requirements must be explicit. Filings and statutory submissions must receive qualified review and approval, and the product must not claim universal global compliance.</t>
+  </si>
+  <si>
+    <t>Functional requirements — planning, treasury, and forecasts
+Purpose: leaders must be able to decide budgets and cash actions from stated assumptions and actual business data. This is a new H4 module using shared controls, records, events, Skills and integration ownership. Depends on E06/E18/E21–E23. It adds Business Budget, Budget Version, Cash Forecast, Scenario, Target and Variance records, separate from platform-spending envelopes. References: the GTM reporting extension and BP's planning, pricing and treasury inventory.
+An owner must be able to set operating targets and approve departmental budgets.
+Budget versions must identify period, currency, assumptions, owner and approval. Actuals and commitments must reconcile to business ledgers.
+Variance alerts must use configured thresholds. Changes must retain history and must not automatically change the AI wallet.
+A treasury owner must be able to inspect cash balances, expected receipts and payments, and runway.
+Forecasts must distinguish cleared, committed, expected and speculative cash and show timing assumptions, foreign-exchange assumptions and stale feeds.
+Scenarios must allow collection, hiring and spending assumptions to change. Any movement of cash must remain a separately approved action.
+A finance leader must be able to compare reproducible forecast scenarios and record a decision.
+Scenarios must use versioned inputs, expose assumptions and sensitivities, and support recommendations with evidence.
+Approval must create owned follow-up work rather than silently reallocating funds.
+An owner must be able to receive a management pack combining financial and operational results.
+Each metric must identify its period, currency, source and freshness and allow drill-down. Narrative must distinguish observed facts from inference.
+Risks and decisions must have owners. Restricted financial information must retain its access controls in Pragya and in exports.</t>
+  </si>
+  <si>
+    <t>Functional requirements — people lifecycle
+Purpose: recruiting, employment operations and exits must remain coordinated and accountable to humans. This is a new H4 domain reusing generic document and channel capabilities and shared platform services. Depends on E01/E03/E05/E06/E07/E09/E11/E26/E28. It adds Position, Requisition, Candidate, Application, Interview, Employee, Employment Agreement, Leave, Payroll Input, Review, Training and Exit Case records. References: BP's people, recruiting, payroll, benefits and training inventory. Full local payroll requires separately validated jurisdiction scope.
+A recruiter must be able to coordinate sourcing, applications, interviews and evidence-based screening.
+Job criteria and screening rubrics must be approved and versioned. Candidate consent and data scope must be recorded.
+Evaluations must cite job-related evidence and uncertainty. Human reviewers must own consequential hiring decisions, while scheduling and communications must reuse governed capabilities.
+A hiring manager must be able to prepare an offer within an approved role and compensation range.
+The requisition, compensation and terms must be checked. Every offer and nonstandard negotiation must receive the assigned human's approval.
+The final agreement must be versioned and signed through E26. Declined or expired offers must not trigger onboarding.
+An employee must be able to complete onboarding, request leave and receive policy answers.
+The employee record must control scoped access. Onboarding tasks must have owners and completion evidence, and leave balances and approvals must follow deterministic rules.
+Answers must cite the applicable policy. HR cases must remain private and escalate when uncertain.
+A payroll or people operator must be able to prepare reviewed payroll inputs and development records.
+Approved hours, leave, compensation changes and reimbursements must reconcile to their sources, with exceptions sent for review.
+Payroll output must target an approved provider or a separately validated local jurisdiction module. Training and appraisals must use transparent criteria and human review.
+An HR owner must be able to execute an approved exit with coordinated access and asset handling.
+The separation decision must be human-authorized. Revocations, asset return, knowledge handover and final-pay inputs must have owners and effective dates.
+Failed or delayed revocation must escalate. Statutory requirements and legal holds must be checked, and completion must be based on evidence.
+An authorized people leader must be able to inspect workforce needs and trends without exposing private records.
+Headcount, capacity, leave and training metrics must obey access and aggregation rules. Predictions must be labelled and must not automatically cause adverse employment action.
+Record corrections and approved exports must be supported.</t>
+  </si>
+  <si>
+    <t>Functional requirements — contracts and obligations
+Purpose: legal and commercial work must move from a request to approved terms, verified signature and tracked obligations. Document generation exists, while contract lifecycle management is a new H4 module. Depends on E03/E05/E06/E09/E11 and shared scheduling, execution and Skill services. It adds Contract, Contract Version, Clause/Playbook, Approval, Signature Envelope, Obligation and Dispute records. References: GTM's proposals and redlines, and BP's legal inventory.
+A contract owner must be able to draft from approved templates and inspect deviations.
+Variables must link to verified business records, and the template and playbook versions must be pinned.
+Comparison and redlines must reveal changed terms and missing information. Liability and nonstandard terms must go to qualified human review.
+An unreviewed legal conclusion must not become an approved clause.
+A legal reviewer must be able to authorize the exact version and signing parties.
+Review must cover commercial authority and exceptions. Edits must invalidate prior approvals where appropriate, and signatory identity and authority must be checked.
+Rejected or outdated versions must not be sent for signature.
+A contract owner must be able to route an approved agreement and verify its execution.
+Creating an e-signature envelope must be idempotent. Signed, declined, expired and provider-pending states must be verified rather than inferred.
+The executed document and signature evidence must be stored. Only verified execution must trigger downstream commitments.
+An obligation owner must be able to monitor renewals, notice dates, duties and disputes.
+Extracted obligations must be reviewable and linked to their clauses. Reminders must have owners and due dates.
+Changes and termination must preserve contract history. Disputes must link relevant support, delivery and finance evidence, and deadlines must not silently lapse.</t>
+  </si>
+  <si>
+    <t>Functional requirements — risk, privacy, and incidents
+Purpose: business obligations, privacy requests and incidents must reach accountable people with reliable evidence. Some platform controls exist, while these H4 business workflows are new. Depends on E01/E03/E05/E06/E07/E09/E12 and independent audit permissions, using shared Skills and controls. It adds Risk, Control, Policy/Obligation, Evidence, Privacy Request, Legal Hold, Incident, Action and License/Insurance Record families. References: GTM's compliance and privacy requirements and BP's risk, incident and corporate-record inventory.
+A risk owner must be able to maintain applicable obligations and an owned control plan.
+Applicability must be reviewed for the supported jurisdiction and sector, including required sustainability or ESG disclosures.
+Each obligation must record source, effective date, owner, evidence and due date. Changes must create reviewed tasks, and monitoring must not imply universal legal compliance.
+An independent auditor must be able to sample controls and track findings.
+Evidence must retain provenance, time, integrity checks, scoped retention and access history. Auditors must not alter the operations they audit.
+Findings must have severity, owner and remediation evidence. Corporate licenses and insurance renewals must receive owned reminders.
+A privacy officer must be able to fulfill a verified person's access, correction or deletion request.
+Identity and request scope must be verified, and relevant business records, conversations, knowledge and derived stores must be enumerated.
+Legal holds must be detected and a reviewer must authorize the actions. Fulfillment must record completion and exceptions and notify downstream systems according to declared responsibility.
+A data owner must be able to understand and govern where business data is used.
+The data map must cover integrations, models, logs, artifacts and backups, with explicit retention, residency and training choices.
+Operational processing consent must not imply model-training consent. Revoked or deleted data must not be silently reused by new learning jobs.
+An incident commander must be able to receive reports from any permitted source and triage, contain and recover a business or security incident.
+Severity, owner, runbook and timeline must be recorded. Safe pre-authorized containment must be deterministic and bounded, and unsafe work must be stoppable promptly.
+Recovery must require evidence and controlled re-enablement.
+An accountable leader must be able to review customer, public and regulatory incident communications and learn from the event.
+Drafts must identify verified facts and uncertainty. Named humans must authorize required communications, and deadlines and delivery outcomes must be tracked.
+Postmortems must assign corrective actions. Deterministic incident status and notifications must remain available when the funded AI reserve is exhausted.</t>
+  </si>
+  <si>
+    <t>Functional requirements — access, assets, and operational maintenance
+Purpose: people and workflows must have the right systems and assets, with predictable maintenance. Some technical tools exist, while business administration is a new H4 module using shared platform services. Depends on E01/E03/E06/E07/E09/E12/E25. It adds Access Request/Grant, Asset, Assignment, Maintenance Plan, Service Ticket and Data Job records. References: BP's IT, facilities and data-pipeline inventory, and GTM's connector-health requirements.
+An IT owner must be able to provision and revoke approved access using least privilege.
+Requests must link to a verified person or role and an approval. Privileged access must receive independent review.
+The target system must confirm granted scopes and effective dates. Failures must remain open, and recertification and exit revocation must retain evidence.
+An operations administrator must be able to track physical and digital assets and recurring maintenance.
+Records must show ownership, assignment, lifecycle, licenses or leases and renewal dates. Planned work must have owners and due dates.
+Overdue maintenance and unused licenses must raise proposals. Purchases and disposals must follow procurement and approval policy.
+A data owner must be able to identify and repair stale or failed business-data flows.
+Freshness and quality checks must link to the relevant jobs and records. Schema changes and reconciliation gaps must create owned exceptions.
+A repair preview must preserve system-of-record rules and idempotency, and reconciliation after repair must demonstrate consistent data.
+A service owner must be able to restore an integration using an approved runbook or a reviewed fix.
+Diagnosis must collect evidence without exposing secrets. Known low-risk runbooks must respect permissions and limits.
+Generated code and adapter changes must enter E32's independent testing and promotion process. Failed repair must escalate instead of repeatedly changing production.</t>
+  </si>
+  <si>
+    <t>Functional requirements — product, experiments, and pricing
+Purpose: the business must turn customer and market evidence into considered product and offer changes. This is a new H4 workflow using shared records, events, Skills, integration ownership and controls. Depends on E06/E13/E18/E19/E24 and E03 for commercial or publishing changes. It adds Idea, Research Finding, Product Requirement, Backlog Item, Experiment, Offer/Price Version and Launch Plan records. References: GTM's voice-of-customer, conversion-optimization and competitive research needs, and BP's product and pricing inventory.
+A product owner must be able to synthesize customer, market and support evidence into a prioritized backlog.
+Findings must preserve source, permission and affected segment. Duplicate requests must consolidate without losing their counts.
+Prioritization must expose impact, effort and uncertainty assumptions. Humans must approve commitments, and customer statements must not become fabricated roadmap promises.
+A launch owner must be able to coordinate an approved product or service release.
+Scope, acceptance, enablement, support readiness, fulfillment and marketing work must have owners. Launch must depend on actual readiness evidence.
+Content and price publication must obey approvals, and rollback and handling of customer impact must be defined.
+An experiment owner must be able to test a hypothesis with agreed measurement and stop rules.
+Population, allocation, success measures, guardrail measures, duration and consent constraints must be explicit.
+Data gaps must be visible, and early stopping and exclusions must be documented. Analysis must not claim causation from unqualified correlations.
+A commercial owner must be able to compare pricing and packaging proposals before applying them.
+Proposals must use cost, demand and contract constraints, with audience, percentage and amount limits and required approval.
+Contractual prices must remain protected. Activated price versions must propagate consistently to quoting and billing and support audited reversal.</t>
+  </si>
+  <si>
+    <t>Functional requirements — partnerships and capital stakeholders
+Purpose: partner, board, investor and corporate-development work must share business evidence under explicit authority. This is a new H4 module reusing research, documents and shared platform services. Depends on E06/E09/E13/E17/E18/E24/E26/E27. It adds Partner Profile, Partner Agreement, Referral, Commission, Stakeholder, Board Action, Diligence Request and Data Room records and reuses Account and Contact. References: GTM's later partner and channel backlog and BP's partnerships and capital inventory.
+A partnership owner must be able to evaluate and onboard a business partner.
+Due diligence, territory, rights, enablement and agreement terms must be recorded, and required review must finish before activation.
+Partner access must expose only shared records. Channel-enablement content must be current and approved.
+A channel manager must be able to track referrals, co-selling and earned commission.
+Referral ownership, deduplication and attribution rules must be explicit. Deal and receipt state must determine eligibility, and disputes must go to review.
+Commissions must reconcile to approved agreements, and payouts must use E22's controls.
+A leader must be able to prepare board and investor reports and retain the decisions that follow.
+Reports must use permissioned, reconciled business metrics and disclose narrative assumptions. External sends must receive named review.
+Meetings must create accepted actions with owners and dates, and confidential strategy must remain separately scoped.
+A capital-process owner must be able to maintain an access-controlled diligence room and research funding or acquisition opportunities.
+Documents must have versions, purpose-limited access and expiry. Requests and answers must have owners, and access and downloads must be audited.
+Research must cite sources. Negotiation and financial commitments must require explicit human authority.
+An executive must be able to delegate scheduling, inbox triage and meeting preparation within explicit boundaries.
+Internal communications must be classified with scoped access. Proposed replies and meetings must use approved channel and calendar controls.
+Conflicts and sensitive requests must route to the owner. Minutes must cite source notes and produce confirmed action items without inventing commitments.
+An owner must be able to turn strategic decisions into owned work and review progress.
+Objectives must link to initiatives, budgets, measurable outcomes and accountable people. Changes must retain the decision rationale.
+Periodic reviews must show actual progress, blockers and assumptions. Cross-functional assignments must require acceptance and must not silently override another owner's authority.</t>
+  </si>
+  <si>
+    <t>Functional requirements — model routing and multimodal work
+Purpose: operators must be able to choose an eligible model or use evaluated automatic selection while retaining quality, policy and cost controls. Vendor adapters and static defaults exist, while dynamic routing and unified asynchronous media jobs are new. Depends on E01/E02/E04/E05/E08/E12 and E32 for learned preferences. D29 defines the required provider catalog, with exact versions and capabilities to be validated during implementation. References: RF §3, §6.4 and §8, RT §§3–5, and the LP and TL defects.
+An administrator must be able to restrict models by capability and data policy.
+The registry must show supported modalities, context limits, tools and approved usage policy. Tenant constraints must filter candidates before selection.
+Pinning an unavailable or ineligible model must cause an explicit failure or a configured eligible fallback. Fallback must never bypass data restrictions.
+An owner must be able to choose Auto and understand its quality and cost tradeoff.
+Routing must consider task class, modality, context, latency, cost ceiling and measured performance, and record the decision and actual cost.
+If no eligible model exists, work must visibly block or enter a declared degraded state. Automatic routing must be tested against the static incumbent before production use.
+An operator must be able to recover from provider failures without repeating business effects.
+Bounded timeouts and retries must distinguish generation from tools that already executed. Fallback must retain context without repeating confirmed effects.
+Cancellation must settle known usage. Provider failures and incompatible tool schemas must produce actionable outcomes.
+A content author must be able to request image, video, editing or audio work and follow progress without blocking other work.
+Jobs must show queued, running, completed, failed and cancelled states, with previews, artifacts and attributed cost. Asynchronous completion must be verified with the provider.
+Unsupported options must fail clearly. Retries must not accidentally charge for or publish duplicate outputs.
+A quality owner must be able to admit or retire models using independent task cohorts.
+Evaluation must measure quality, tool and schema accuracy, cost, latency and policy compliance. Changed model versions must have regression evidence, rollback and reporting of affected workflows.
+Benchmark scores alone must not enable production use.
+A voice or media owner must be able to select a provider validated against the actual language, interruption, tool, latency and artifact requirements of a supported use case.
+Quality thresholds must be agreed per use case. Mid-call failure must follow a tested transfer or closure plan, and every new provider must pass capability-specific acceptance.
+An administrator must be able to enable validated adapters and capability profiles for Gemini, Claude, OpenAI, GLM, Qwen and Kimi.
+Credentials must be tenant-scoped. Model and version, region, modality and data-policy constraints must be explicit, and unavailable providers must fail clearly rather than being implicitly selectable.
+A content owner must be able to use the supported video capabilities for Veo, Seedance and Wan, with asynchronous status, cancellation, policy checks, usage attribution, persistent artifacts and duplicate-publication protection.
+The supported image catalog must include Gemini Image, GPT Image, Qwen Image and Kling with capability-specific options, safety checks, previews, artifacts, cost attribution and deterministic failure handling.
+Unsupported image-option combinations must be rejected before spending.
+A platform owner must be able to replace or add a model without rewriting business workflows.
+Adapters must implement a common contract. Version pinning, fallback eligibility, routing decisions, migration and rollback must all be recorded.</t>
+  </si>
+  <si>
+    <t>Functional requirements — evaluated learning and self-improvement
+Purpose: improvements must earn deployment through evidence and remain reversible. Memory, reflection and Board machinery partly exist with integration defects, while the complete promotion cycle is new. Depends on E02–E05, E08, E12 and relevant business metrics. Decisions D15 and D23 require independent evaluation and authorized promotion rather than self-approval or calendar-based improvement claims. References: SK §11, GTM §11, RF §§5, 10 and 12, RT §§7, 9 and 22, and the MI, MC and PC defects.
+A quality owner must be able to link human feedback and business outcomes to the versions that produced them.
+Run, Skill, model and policy versions must link to success, edits, rejections, complaints, cost and delayed outcomes. Missing labels must remain unknown.
+Feedback must obey consent and access restrictions, and metrics must support comparisons between equivalent cohorts.
+A workflow owner must be able to assess a candidate before replacing the incumbent.
+Independent curated cases and reference cases from the incumbent must include negative and adversarial scenarios. Skipped tests or exhausted test budgets must not count as passes.
+Human spot checks must supplement automated scoring. The report must show regressions and changes in cost and latency.
+A capability owner must be able to turn repeated successful work into a reusable Skill proposal.
+The proposal must link observed patterns and examples, define scope and proposed scripts or instructions, and check for existing reusable work before creating a duplicate.
+The candidate must pass E08's authoring requirements and E32's evaluation and remain inactive until promotion is authorized.
+A workforce owner must be able to test and adopt improved instructions or routing preferences.
+The proposal must state evidence and expected benefit. An approved limited rollout must compare the candidate with the incumbent under bounded exposure.
+Predefined regression rules must automatically restrict or roll back the change. Original versions and decisions must remain auditable, and improvement must not be guaranteed merely because time has passed.
+A service owner must be able to request a missing or repaired capability without allowing unreviewed changes to live behavior.
+Generated code must execute only in the approved isolated runtime and undergo independent tests, permission checks, metering and adversarial checks.
+Ordinary tenant Skills must not rewrite sensitive primitives. The exact changes and their impact must be presented for independent human approval.
+An operator must be able to promote or roll back a reviewed capability safely.
+The promoter must be distinct from the author or proposer. The active-version change must be atomic, distributed workers must converge on it, and handling of in-flight runs pinned to prior versions must be explicit.
+A failed limited rollout must disable affected effects and restore a known version. Since rollback cannot undo real-world effects, it must create reconciliation tasks where required.</t>
+  </si>
+  <si>
+    <t>Functional requirements — Generative and adaptive experience
+Purpose: a new frontend must help people operate their business through appropriate conversational and structured views. This is new work, while the current frontend must remain usable in earlier releases. Depends on the supported capabilities' APIs and authorization, E10's Pragya flow and E06's schema metadata. D05 requires an explicit Design Gate before implementation, D26 makes Pragya the single human workspace, and D31 requires the digital-twin experience developed with E39/E40. References: RF §11, RT §8 and the confirmed product decisions.
+A product owner must be able to approve a complete experience direction before frontend development starts.
+Design and brainstorming must cover owner, operator, reviewer and administrator journeys, information architecture, interaction prototypes, visual language, accessibility, mobile behavior and failure states.
+Review must test realistic work and record decisions. Implementation of the new frontend must wait for explicit design acceptance.
+A reviewer or operator must be able to understand how generated views retain user control.
+Prototypes must demonstrate record detail and editing, activity feeds, approvals, budgets, workflow configuration and handoff to Pragya.
+Consequential actions must have stable, discoverable controls. Unsupported generation must have a usable fallback, and research must measure comprehension as well as appearance.
+A user must be able to receive a task-appropriate view and retain a preferred arrangement.
+Generated view definitions must select approved components and validated data bindings. Backend authorization must govern every data and action request.
+Generated views must not introduce arbitrary executable UI code or grant additional access. Preferences must be editable and resettable, and stale or incompatible schemas must produce a useful recovery state.
+An existing user must be able to move to the new frontend without losing essential workflows.
+The parity checklist must include authentication, records, execution, artifacts, approvals, integrations, budgets and account administration.
+Migration must be staged, monitored and reversible. The current UI must remain available until its replacements pass, and accessibility and task success must be measured.
+The Pragya workspace must support voice-first interaction alongside text, direct visual edits, analytics drill-down and immediate stop.
+The experience must include a detailed isometric 3D digital twin and a knowledge and assets explorer. It must show available levels first, with a usable accessible alternative.
+Persisting all six organizational levels must depend on the optional E40 Graph/Loop capability rather than inventing a mandatory legacy hierarchy.</t>
+  </si>
+  <si>
+    <t>Functional requirements — product packaging and organizational scale
+Purpose: a business must be able to adopt useful workflows progressively and expand its organizational scope safely. Tenant and partner hierarchy exist, while modular packaging and business-unit governance are new. Depends on E01/E04/E06/E09/E12 and the capabilities included in each package. D01 rejects inherited bundle and agent counts, while D32 supports ad hoc work alongside Solo, MSME, startup and enterprise package candidates whose contents and prices remain open. References: GTM's tenant-zero and commercial questions, useful adoption and scale needs from BP, and the product decisions.
+A buyer must be able to understand the outcomes a package supports and the prerequisites it needs.
+Each package must identify supported workflows, integrations, required human roles, autonomy, limitations and usage estimates.
+A fixed agent count must not be the value promise. Activation must check prerequisites and create only the needed configurations, and failed setup must remain recoverable.
+A commercial owner must be able to price and support a package using measured economics.
+Tenant-zero evidence must include actual workloads, outcomes, variable costs, idle storage costs, reviewer effort and support burden.
+The commercial model and free allowance must be explicitly chosen under O04. Unapproved per-seat or per-outcome prices must not be treated as settled decisions.
+Plan changes must preserve entitlements and records. A finite ad hoc task must not require activation of an entire business package.
+A group owner must be able to manage business units with different budgets, policies and data access.
+Parent visibility must be explicit. Approved policies must inherit downward and metrics aggregate upward, with no default sharing between siblings.
+Storage and processing placement must actually satisfy model and residency requirements. Separate legal entities and currencies must not be combined into misleading totals.
+A partner administrator must be able to support assigned businesses within their boundaries.
+Assignments and delegated roles must determine access. Pricing and branding privileges must be bounded, and support actions must identify the actor in the audit trail and use time-limited access where appropriate.
+Tenant offboarding must revoke delegation and preserve the tenant's export rights.</t>
+  </si>
+  <si>
+    <t>Functional requirements — BabyBuddha and OmniBuddha research
+Purpose: in-house models may be used if comparative evidence shows better task quality or lower cost. This is a research aspiration, not a shipped capability, an approved investment or a prerequisite for the business product. Depends on E31/E32 and explicit permission to use data. H6 is an investment decision rather than a promised launch. References: RF §3.1 and §8.1, and RT §§3 and 5.
+A data owner must be able to choose whether eligible traces can be used in model development.
+Explicit opt-in must record the permitted purpose and data categories. Tenant-secret and personal-data restrictions must apply, and withdrawal must stop future collection within that scope.
+Data lineage and retention must be reviewable. Operational memory must not be treated as implied training consent.
+A research sponsor must be able to decide whether post-training an open-weight model is worthwhile.
+The research proposal must document licensing and serving constraints, the approved dataset, incumbent baselines, task cohorts and full cost.
+Evaluation must compare tool use and reasoning, or multilingual speech quality, as appropriate. Evidence must determine whether research continues or stops.
+A model owner must be able to propose BabyBuddha for eligible text and tool workloads.
+Fast and reasoning profiles must pass independent quality, safety, tool-reliability, latency and cost checks against the incumbent.
+A limited rollout and eligible fallback must exist. Without sufficient evidence, current providers must remain the default.
+A voice owner must be able to propose OmniBuddha for a validated speech workload.
+Tests must cover supported languages, switching languages within a conversation, interruption, tool calls, consent handling, latency and funded safe closure.
+Failed calls must have tested handoff or termination behavior. Production admission and rollback must use E31/E32's controls.</t>
+  </si>
+  <si>
+    <t>Functional requirements — isolated relational tenant data plane
+Purpose: every tenant must have a queryable, exportable relational business database, and no tenant may access another tenant's business payload. Shared models and operational tables exist, but the isolated relational data plane is new. Depends on E01/E02/E03/E04/E06/E07/E09/E12. Decisions D02, D09 and D25 confirm typed relational storage and the shared-control-plane boundary. References: the tenant and ad hoc backlog, the operating model and product decisions.
+A tenant must be able to store business records in a dedicated relational database.
+The database must use typed tables, foreign keys, constraints, indexes and reviewed versioned migrations.
+Campaigns, contacts, activities, finance and other module records must be queryable without a generic JSONB record store or JSONB custom-field bag.
+A Skill or application must be able to use a safe tenant data API.
+Every request must be tenant-scoped and authorized. Filtering, sorting, pagination, transactions, validation, optimistic concurrency and audit attribution must be defined.
+Cross-tenant identifiers and unbounded queries must fail safely. Skills, agents and applications must use the tenant API or record service for business-state access.
+A platform owner must be able to keep only the agreed metadata in shared services.
+The shared control plane must hold identity and login, subscriptions, billing, and minimal routing and accounting metadata.
+Business records, detailed execution payloads, files, Cortex, code, applications and websites must remain in the isolated tenant environment.
+Data placement must be visible in architecture documentation and access tests. Multiple private containers or volumes may serve a tenant, but the database lifecycle must remain independent of an idle-paused code process.
+A GTM operator must be able to use one tenant-owned history for campaigns, leads and calling.
+Existing campaigns, campaign_calls, lead_queue and related lead, contact and calling data must migrate into typed tenant tables aligned with E13–E18.
+Identifiers, statuses, timestamps, consent, recordings and references, and outcomes must be preserved. The old shared path must be removed after verified cutover.
+A security owner must be able to prove tenant isolation across APIs, tools, workers, event consumers, scheduled jobs, logs, caches, volumes and network policies.
+Negative tests must prove that a tenant cannot address another tenant's records or files. Resource and storage limits must be enforced.
+An owner must be able to recover or leave with the complete business state.
+Export and restore must include the tenant database and artifact, source-document, Cortex and application manifests, together with permitted control metadata.
+Checksums, schema version, permissions and restoration evidence must be recorded, and restoration must not expose data to another tenant.</t>
+  </si>
+  <si>
+    <t>Functional requirements — tenant runtime, generated software and hosting
+Purpose: a tenant must be able to create and operate generated tools, internal applications and websites within its own isolated runtime. Depends on E01/E02/E03/E04/E08/E09/E12/E36, with generated-code promotion governed by E32. Tenant-local placement follows D25 and solution design follows D30. References: the tenant and ad hoc backlog and the operating model.
+A tenant must be able to run generated code and tools without gaining host access.
+Tenant containers must use versioned runtime images, isolated processes, network and credential policies, CPU, memory and time limits, and metering.
+Workers must never silently fall back to host filesystems or credentials.
+A capability owner must be able to reuse generated code safely.
+Source code, dependencies, tests, configuration references and build provenance must be stored in tenant-local versioned repositories.
+Workers must reload pinned versions. Changes must be reviewed, evaluated, promoted and rolled back through E32.
+An owner must be able to request an internal app for a business need.
+The request must become a tenant-local specification covering data tables and APIs, UI, workflows, permissions, limits and acceptance tests.
+The app must be previewable, editable and versioned before deployment.
+An administrator must be able to operate an app under the same platform controls as other work.
+App requests must use the tenant API and approved Skills or tools. Deployments must be isolated, observable, cancellable and auditable.
+Upgrades and rollback must preserve records and handle active-run behavior correctly.
+A tenant must be able to build, preview and host a website.
+Source, assets, builds, preview URL and publication state must be tenant-owned. Provider and domain configuration must be explicit and portable.
+Publication must require permissions, safety checks and a rollback capability.
+An operator must be able to find and manage source mirrors, uploads, artifacts, code, apps and site builds in stable tenant-storage folders.
+File metadata must include owner, provenance, version, retention and checksum. Quotas, alerts, deletion and restore must be enforced.</t>
+  </si>
+  <si>
+    <t>Functional requirements — Cortex knowledge graph and legacy RAG retirement
+Purpose: tenant agents must use traceable, editable knowledge and procedural memory built from original source material. The new Cortex path must replace the legacy document-ingestion and RAG implementation. Depends on E01/E02/E05/E06/E09/E10/E12/E36/E37. D27 defines acquisition and cutover, with D25 keeping the data tenant-local. References: the tenant and ad hoc backlog, product decisions and the source-coverage review.
+A new tenant must be able to teach the system about the company in a clear sequence.
+Registration must trigger bounded research of the company website, followed by requests for relevant uploads and connections to Google Drive, OneDrive, SharePoint and other approved sources.
+Pragya must show progress, consent, scope and failures.
+A tenant must be able to keep original files unchanged and mirror updates predictably.
+Originals must be saved in tenant folders with source URI, path, version, checksum, timestamps and synchronization cursor.
+Resynchronization, renaming, deletion and permission changes must be represented without silently overwriting provenance.
+An operator must be able to inspect and edit the tenant knowledge graph.
+Entities, relationships, procedures, assumptions and confidence must link to exact source documents and locations.
+Edits must retain version, author and reason. Retrieval must be tenant-scoped and permission-aware.
+An agent must be able to use Cortex evidence during work.
+Skills must receive citations, provenance, freshness and access decisions. Conflicting or missing evidence must be surfaced for review.
+Procedural updates must be testable before they affect approved workflows.
+A platform owner must be able to retire the legacy document-ingestion and RAG implementation completely.
+The migration must inventory old document and chunk tables, endpoints, jobs, indexes and flags, and move the required evidence into Cortex.
+After cutover, no production path may read or write the legacy store. Old code and tables must be removed, except for an explicitly isolated legal archive where required.
+Extraction and search must remain capabilities of the new Cortex path, with no parallel legacy RAG store or live dual-write path.
+An operator must be able to verify that cutover preserved the required knowledge.
+Replay and comparison must prove source coverage, links, permissions and retrieval behavior. Dashboards must identify orphaned originals and originals that have not been ingested.
+Rollback must be limited to versions of the new Cortex implementation and must not re-enable the retired RAG path.</t>
+  </si>
+  <si>
+    <t>Functional requirements — Pragya solution design and ad hoc workbench
+Purpose: Pragya must be the single human workspace for packaged business operations and finite, one-off work, with every new solution designed collaboratively before deployment. Depends on E03/E05/E07/E08/E10/E12/E31/E33/E36/E38. D26 confirms voice-first operation with text and visual controls, D30 requires a shared solution blueprint and D32 confirms ad hoc work without mandatory pack activation. References: the tenant and ad hoc backlog, the operating model and product decisions.
+An owner must be able to describe a finite business goal outside a standard package.
+Pragya must accept the goal, constraints, source data and desired outputs and propose a bounded one-off plan.
+The task must not require a permanent agent hierarchy or activation of a Solo, MSME, startup or enterprise pack.
+An analyst must be able to turn raw data into a defensible financial model, market study or presentation.
+The run must select approved Skills, models and tools, record assumptions and calculations, cite evidence and produce editable artifacts.
+Material uncertainty and external effects must receive the required review.
+A tenant must be able to brainstorm a proposed solution with Pragya before deployment.
+A full solution-architect Meta Agent must turn the conversation into an editable blueprint covering goals, users, records, Skills and tools, integrations, events, schedules, permissions, budgets, risks, tests and success measures.
+Unresolved assumptions must remain visible.
+The tenant and Pragya must be able to edit the same design without losing decisions.
+Voice, text and visual controls must edit one versioned specification, with near-real-time presence and conflict handling.
+Changes must show authorship, differences, conflicts and approval state. Deployment must remain blocked until required reviewers approve the blueprint.
+A human operator must be able to access supported business functions through one workspace.
+Pragya must support voice-first and text interaction, contextual visual controls, generated analytics and drill-down.
+Every action must still use authorized platform APIs or Skills and retain audit history and provenance.
+An operator must be able to stop unsafe work immediately through a prominent, authenticated control.
+Stop must revoke eligible execution, prevent queued effects, settle known usage and show deterministic status.
+The stop control must work when voice, a model or a secondary channel is unavailable.</t>
+  </si>
+  <si>
+    <t>Functional requirements — optional Graph/Loop operating model and digital twin
+Purpose: tenants that need organizational modeling must be able to traverse and operate a Graph → Loop → Process → Agent → Skill → Action structure. Graph and Loop are optional, and ordinary workflows must remain valid without them. Depends on E03/E06/E07/E08/E10/E31/E33/E39. D07 defines the optional hierarchy and D31 defines the digital-twin experience, with E33's Design Gate preceding the new frontend. References: the tenant and ad hoc backlog and product decisions.
+An owner must be able to model the whole business as an optional Graph, with each Loop representing a department or function.
+Processes must retain their workflow meaning, Agents their role meaning, Skills their reusable-capability meaning, and Actions their tool-wrapper meaning.
+Every node must have a version, owner, policy, budget and data scope.
+An administrator must be able to validate and compile the hierarchy into executable work.
+References must resolve to versioned Skills and Actions. Permissions, budgets, memory scope, schedules and event subscriptions must be checked before activation.
+Cycles, duplicate ownership and unresolved nodes must fail with actionable diagnostics.
+An owner must be able to zoom from the business overview to an individual action through the new frontend's isometric digital twin.
+The view must traverse Graph, Loop, Process, Agent, Skill and Action where enabled and show dependencies and live status.
+The organizational Graph must be clearly distinguishable from a workflow dependency graph and the evidence-based knowledge graph. Available levels must be shown without forcing the optional hierarchy on every tenant.
+An operator must be able to edit the model visually and inspect its evidence.
+Visual editing must use the same versioned blueprint as Pragya, show the impact on permissions, budgets and runs, and link analytics to tenant records and source documents.
+An accessible alternative to the 3D view must be available.
+A business owner must be able to add or reorganize departments without duplicating execution.
+Adding or removing Loops must recompute routing, policy inheritance, budgets and reporting. Existing runs must retain their pinned versions, and event and schedule subscriptions must remain idempotent.
+A tenant without the hierarchy must still be able to run flat Process, Agent, Skill and Action workflows and ad hoc jobs with equivalent authorization, observability and stop controls.
+Enabling the hierarchy must be reversible and must not copy executable Skill versions or require extra model calls at every organizational level.</t>
   </si>
 </sst>
 </file>
@@ -7393,7 +8080,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="59" spans="1:17" ht="51" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:17" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>55</v>
       </c>
@@ -8413,7 +9100,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:17" ht="51" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>75</v>
       </c>
@@ -11374,7 +12061,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="138" spans="1:17" ht="63.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="10">
         <v>134</v>
       </c>
@@ -11425,7 +12112,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="139" spans="1:17" ht="63.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="10">
         <v>135</v>
       </c>
@@ -11476,7 +12163,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="140" spans="1:17" ht="63.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="10">
         <v>136</v>
       </c>
@@ -11527,7 +12214,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="141" spans="1:17" ht="63.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="10">
         <v>137</v>
       </c>
@@ -14292,7 +14979,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="196" spans="1:17" ht="63.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" s="14">
         <v>192</v>
       </c>
@@ -14341,7 +15028,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="197" spans="1:17" ht="63.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="14">
         <v>193</v>
       </c>
@@ -14390,7 +15077,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="198" spans="1:17" ht="63.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="14">
         <v>194</v>
       </c>
@@ -14439,7 +15126,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="199" spans="1:17" ht="63.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="14">
         <v>195</v>
       </c>
@@ -16292,7 +16979,7 @@
         <v>1242</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+    <row r="9" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
         <v>238</v>
       </c>
@@ -16305,32 +16992,11 @@
       <c r="D9" s="26">
         <v>1</v>
       </c>
-      <c r="E9" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — Skills and controlled capabilities
-Purpose: reusable business capabilities must be authored as Skills, with controlled tools enforcing their effects. The Skill tier and some dynamic-tool code exist, but the version and asset model is new. Depends on E01–E05 and E12's sandbox controls. Decision D04 confirms Skills as the main authoring unit. References: SK throughout, GTM §6, FEAS N-6/N-7, and the TL, EP and MI defects.
-A Skill author must be able to create a reusable capability with instructions, input and output contracts, scripts and assets.
-Database-backed drafts must describe their purpose, discovery information, permitted primitives, governance and runtime reference.
-Published versions must be immutable, with working comparison, testing, publication and rollback. Each execution must pin and record its chosen version.
-A workforce designer must be able to reuse a Skill without adding unnecessary agent reasoning loops.
-Eligible Skills must first expose brief metadata, with full instructions loaded when selected. Selection must respect access and suitability for the task.
-Direct invocation and optional Action wrappers must both work. Multiple consumers must be able to share one version without indiscriminately copying ownership or memory.
-A tenant administrator must be able to run authored scripts without exposing credentials or the host environment.
-Approved runtime images must supply dependencies. Assets must be verified by hash and isolated by tenant, version and run where needed.
-Authored code must not install packages at runtime or fall back to host execution. Resource, network and file limits must be enforced, and external credentials must remain behind controlled tools.
-An operator must be able to enable a capability once and use it across workers and restarts.
-Registry entries must resolve to executable implementations, and workers must reload the correct version of each tenant capability.
-Discovery and execution must both check tenant, enabled status and permissions. Disabling a capability must take effect everywhere, and unknown definitions must not execute.
-An operator must be able to generate documents reproducibly through the reference Skill family.
-Deterministic DOCX, PPTX, PDF and spreadsheet boilerplate must become stored scripts and assets, while prompts retain work requiring judgment.
-Outputs must be registered artifacts. Tests must compare quality, token use, latency and cost with the existing path, and attribute usage to the Skill version and sandbox.
-A capability owner must be able to consolidate social and integration wrappers without losing controls.
-Selected operations must be piloted through authenticated controlled primitives and platform Skills, retaining operation permissions, consent, idempotency and budgets.
-Migration must compare task quality and cost, support rollback, and retire old paths only after a verified cutover.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E9" s="28" t="s">
+        <v>1244</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
         <v>268</v>
       </c>
@@ -16343,35 +17009,11 @@
       <c r="D10" s="26">
         <v>1</v>
       </c>
-      <c r="E10" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — connections and system-of-record sync
-Purpose: connecting an external system must produce usable, recoverable capabilities with clear data ownership. Some adapters exist, while MCP transport and complete synchronization are new. Depends on E01, E03 and E08, and on E06/E07 for record synchronization. Under D02, hybrid mastering and HubSpot as the first reference connector remain proposals requiring confirmation. References: GTM §§4 and 7, FEAS N-6, RT §21, and the TL defects.
-An administrator must be able to connect, test, rotate credentials for, and revoke an external service.
-Setup must show supported operations and scopes, the connected account, test results, health and limits.
-Credentials must be encrypted and excluded from model prompts. Expired tokens must produce an actionable reconnect state.
-Revocation must disable dependent effects and identify the workflows affected.
-An administrator must be able to attach an approved MCP server and use its permitted capabilities.
-The chosen transport must work end to end, and saved configuration must reconnect on every worker.
-Discovering a tool must not itself grant permission to execute it. Server metadata must be treated as untrusted, with explicit operation policies and limits applied independently.
-Timeouts, outages and revocations must have visible outcomes.
-A CRM owner must be able to declare the authoritative system for each object and trust the local mirror.
-External identifiers, field mappings and freshness must be visible. Writes to externally mastered records must wait for confirmed write-back.
-Conflicts must preserve the losing change for review. Retries and webhook replays must neither duplicate records nor cause changes to oscillate between systems.
-An owner must be able to move an object deliberately between local and external mastering.
-Migration must preview affected records, relationships, consent and conflicts, preserve a recovery snapshot, backfill mappings, reconcile counts and obtain required approval.
-Partial failures must support resumption or rollback. A connector outage must never silently change the authoritative system.
-A business user must be able to synchronize the knowledge and collaboration sources their workflow needs.
-Drive, SharePoint, Notion, Slack and Teams must be prioritized according to the chosen pilot. The Cortex acquisition path must also support the approved OneDrive scope described in E38.
-Synchronization must respect source permissions, changed and deleted documents, and progress cursors. Review cards must use the same authenticated approval service as other interfaces.
-Every advertised integration must pass a representative end-to-end use case.
-An administrator must be able to distinguish available, preview, unavailable and planned capabilities in the integration catalog.
-The catalog must cover calendar, email, CRM, analytics, enrichment, e-signature, payments, bank feeds, tax, HRIS, inventory and helpdesk families.
-Enabling an integration must require evidence that connection, metering, policy enforcement and recovery work.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E10" s="28" t="s">
+        <v>1245</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
         <v>298</v>
       </c>
@@ -16384,33 +17026,11 @@
       <c r="D11" s="26">
         <v>3</v>
       </c>
-      <c r="E11" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — Pragya and business onboarding
-Purpose: an owner must be able to turn business goals into a reviewable operating setup and supervise it through Pragya. This is a new experience built on partial entity-builder and Board capabilities. Depends on E01, E03, E05 and E08, and E06/E09 for connected operations. Decisions D26 and D30 establish Pragya as the single, voice-first human workspace and require collaborative solution design. References: RF §§4–5, GTM §11, RT §11, and the MI defects.
-A new owner must be able to establish business context without answering questions the product can already resolve.
-Pragya must research supplied and public sources, show its assumptions, ingest approved internal sources and revise conclusions with provenance.
-It must ask only unresolved questions and must never save a speculative business fact as verified. Discovery must support pausing and resuming.
-An owner must be able to agree workflows, intended outcomes and boundaries before deployment.
-Planning must capture business problems, owners, priorities, KPIs, budgets, data and mastering choices, permitted channels and review rules.
-The proposal must identify required Skills, integrations and missing capabilities, with changes available for review. A Solo Pack or fixed agent roster must not be mandatory.
-A designer must be able to request a capability and receive an editable, tested candidate.
-The builder must look for reusable capabilities before creating new ones and must be able to revise failed candidates.
-Tests must include independent known cases, failures and permission boundaries. Skipped tests and tests stopped by an exhausted budget must not count as passes.
-Generated work must remain a draft until an authorized person promotes it.
-An owner must be able to preview a business workflow realistically before activating it.
-The preview must show representative inputs and outputs, approval points, records affected, dependencies and estimated costs without causing live effects.
-Missing credentials or policies must block activation. Deployment must use pinned versions and the chosen autonomy policy.
-An owner must be able to ask what happened, what needs attention and what it cost.
-Pragya must answer from actual records and runs, link the evidence, distinguish observed results from estimates, and show pending reviews, failures and business outcomes.
-Requested changes must pass the same permissions and approval controls as direct UI actions.
-An owner must be able to continue through voice, text or a verified collaboration channel, with channels introduced only when their adapters have demonstrated readiness.
-Authorized identity and permitted context must survive handoff. Private reports must not reach external counterparties, and unverified or sensitive requests must receive the required verification.
-A failed channel must offer a valid fallback. Text, directly editable views and immediate stop controls must remain available within the Pragya workspace.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E11" s="28" t="s">
+        <v>1246</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>328</v>
       </c>
@@ -16423,40 +17043,11 @@
       <c r="D12" s="26">
         <v>1</v>
       </c>
-      <c r="E12" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — Karuna and communication channels
-Purpose: customer-facing interactions must share conduct rules, identity, history and escalation behavior. Voice, email and messaging paths exist with major gaps. Depends on E01–E05, E07–E09 and E06's consent and activity records. D03 requires an approved workflow policy for routine effects, exception and mandatory-checkpoint review, and an explicit session policy for live voice. D06 requires funded safe closure without intentional debt, and D28 requires complete Exotel integration. References: GTM §§3, 8 and 11, FEAS §§2–4, BP §2.3, and the VT, GW and TL defects.
-An owner must be able to enforce contact permission and conduct before every external action.
-Email, calling, messaging, social, browser and connector paths must check consent and purpose, suppression, recipient or account ownership, time windows, disclosure policy and required human review immediately before execution.
-Policy failure must block the action, and prompts must not override it.
-A customer must be able to set contact preferences, stop contact and request a human.
-Opt-out must promptly update shared suppression and stop queued and future prohibited contact. Verified preferences must apply across linked channels.
-A human request must create an owned handoff. If nobody is available, the customer must receive an honest callback or response expectation.
-An operator must be able to run inbound and outbound voice under an approved session policy.
-Carrier routing, recording and disclosure choices, interruption, tool calls, costs, disposition and activity linkage must work end to end.
-Consent and funds must be checked before dialing, every tool effect must use platform controls, and safe closure must be funded in advance. Low credit or an outage must not cause intentional debt.
-An operator must be able to handle email, messaging and web conversations through a coherent inbox showing threads, participant identity, attachments, delivery state and assignment.
-Reconnects and retries must not duplicate sends. Uncertain delivery must not be reported as successful.
-Handoffs must carry permitted history without exposing private operator conversations.
-A customer must receive appropriate communication in a supported language, following brand tone and accessibility rules.
-Language detection and translation must disclose uncertainty and preserve material meaning. Unsupported languages must route to help.
-Persona settings must affect delivery without promising a guaranteed emotional response from a numeric setting.
-An operator must be able to recover from a channel outage while respecting the fallback channel's consent and customer preferences.
-Queued work must retain ordering and stop rules. Callback promises must create owned tasks.
-Real-time streams must be authenticated and resumable where possible. Failed sessions must preserve trustworthy cost and outcome records.
-An owner must be able to connect Exotel for approved calling use cases with tenant-scoped credentials, verified account and number ownership, signed webhooks, regional settings, and recording and disclosure policy.
-Connection health and capability limits must be visible. Unsupported use cases comparable to Smartflo must fail clearly.
-Exotel inbound and outbound setup, answer, busy, no-answer, failure, transfer, hangup and human handoff must map to durable call and activity records.
-Consent, suppression, schedules and funds must be rechecked immediately before dialing.
-Signed callbacks must be reconciled idempotently. Delayed, duplicate and out-of-order events must not move a call back to an earlier state.
-Recording references, consent, retention and access must be stored in the tenant data plane, with unknown outcomes surfaced for review.
-Timeouts, rate limits, provider outages and missing webhooks must trigger bounded retry and reconciliation without blind redial or duplicate business effects.
-Metered costs and closure reserves must settle accurately, and fallback and emergency-stop behavior must be tested.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E12" s="28" t="s">
+        <v>1247</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
         <v>372</v>
       </c>
@@ -16469,37 +17060,11 @@
       <c r="D13" s="26" t="s">
         <v>1191</v>
       </c>
-      <c r="E13" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — operational readiness and service continuity
-Purpose: the product must be demonstrable, releasable, recoverable and supportable with evidence. The application exists with substantial release and operational defects. This work is cross-cutting and must be delivered alongside the capabilities it protects. D25 defines tenant-data placement, and D33 requires defects to be revalidated rather than assumed closed by replacement. References: DR, the FE, TS, IN, SA, DM and API registers, and GTM §4.2.
-A developer must be able to start a fresh local checkout without production domains or credentials.
-The supported environment, dependencies, migrations and fixtures must be documented. Local URLs must be explicit, and missing configuration must never default to production.
-Mock and offline tests must be distinguishable from live-provider tests. Public callback setup must be separate from basic local operation.
-A release owner must be able to establish that required checks actually ran.
-Continuous integration must trigger for active backend and frontend paths and report executed counts for required unit, integration, UI and regression tests.
-Missing infrastructure must fail required checks. Security and tenant isolation, approvals, money and replay scenarios must exercise real dispatch paths, and documentation must identify unverified services accurately.
-An operator must receive useful error, loading, empty and permission states, reconnect guidance and actionable request identifiers.
-Metrics must expose policy failures, queue age, approvals, cost mismatches, connector health and run outcomes. Log access must be scoped and secrets redacted.
-A tenant owner must be able to recover or export the complete supported business state.
-Encrypted automated backups must begin before operational writes. Restore drills must include record versions and relationships, knowledge, memory, configuration, relevant history and ledgers, and artifact manifests.
-Exports must be usable and tenant-scoped, exclude raw credentials and identify missing external data. Recovery and acceptable data-loss targets must be agreed and measured.
-A service owner must be able to operate tenant databases independently of code execution.
-Database sleep and startup, connection pools, durable volumes, upgrades, capacity and backups must have explicit lifecycle controls.
-Work must park when its tenant database is waking or unavailable. Readiness must be monitored per tenant, and persistent storage must not depend on local scratch directories.
-A product owner must be able to decide whether a release is supportable.
-Every enabled capability must have a supported-version record, an owner, a rollback procedure, an operating runbook and acceptance evidence.
-Blockers and unresolved defects must be explicit. Unsupported tools must be inaccessible, and superseded runtime paths must be removed after verified migration and the defined rollback-retention period.
-Before work starts in an area, its numbered defect register must be checked against the current code and runtime path.
-Each item must be classified as applicable-repair, replaced-path, not-reproducible, deferred or accepted-risk, with evidence, an owner and a date. Duplicate identifiers must remain cross-referenced without double counting.
-Applicable T0 and T1 defects must become release-blocking stories or tests in the responsible epic.
-Fixes must be verified through API, worker, tool, UI and external-provider paths where relevant. Feature flags and seed data must not count as proof, and missing infrastructure must not allow tests to pass by silently skipping.
-Closing a defect must link the change, regression evidence and current behavior. Replacing a component must not automatically close its defects.
-Deferrals must record the reason, mitigation and review date. Unresolved defects must remain visible in release readiness and must not be relabelled as completed features.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E13" s="28" t="s">
+        <v>1248</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
         <v>413</v>
       </c>
@@ -16512,32 +17077,11 @@
       <c r="D14" s="26">
         <v>2</v>
       </c>
-      <c r="E14" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — market intelligence and targeting
-Purpose: marketing and sales teams must build a defensible understanding of markets, accounts and audiences. Research and artifact tools exist, while durable business intelligence is new. The primary operators are marketing and revenue operations. Depends on E01–E05 and E08, with E06 for records, E07 for monitoring, E09 for connected sources and E11 for any external communication. References: GTM §§6 and 9, and FEAS §2.
-A marketer must be able to produce a cited company, market or competitor brief through a reusable Skill.
-Findings must identify their source and observation date, distinguish claims from inference, and flag inaccessible or conflicting evidence.
-The brief must be downloadable without being published externally.
-A marketer must be able to monitor news, pricing and feature changes, hiring, funding, reviews and category developments without repeated alerts for the same observation.
-Scheduled research must compare new observations with prior records. Deduplication must retain provenance, and meaningful changes must create owned Business Signals.
-Unknown data must not become a fabricated trend.
-A revenue owner must be able to define and revise an ideal customer profile with explainable scoring.
-Rules, weights and disqualifiers must be versioned. Scores must show supporting evidence and missing fields.
-A revised definition must support rescoring a preview cohort before activation. Enrichment must obey restrictions on protected and sensitive data.
-A seller must be able to build target-account and buying-group lists from permitted evidence.
-Account and contact enrichment must record source, freshness and confidence. Identity deduplication must use E06, and saved segment criteria must reproduce the same selection logic.
-Finding contact details must never imply permission to contact. A vendor enrichment service must be replaceable behind the same Skill contract.
-A seller must be able to prepare account briefs, competitive battlecards and evidence for responding to objections.
-Outputs must use the current approved messaging library and cite sources, mark unsupported comparisons, and restrict sensitive customer evidence to permitted users.
-The brief version must link to the relevant account or deal.
-An owner must be able to turn an insight into a proposed campaign, account task, risk or product idea and later assess its value.
-The receiving owner must accept or reject the proposal with a reason. Resulting work and outcomes must link to the original insight.
-Read-only research must not silently trigger an external send.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E14" s="28" t="s">
+        <v>1249</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
         <v>444</v>
       </c>
@@ -16550,31 +17094,11 @@
       <c r="D15" s="26">
         <v>2</v>
       </c>
-      <c r="E15" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — content and demand generation
-Purpose: a brand owner must be able to move from evidence-backed briefs to reviewed assets, publication and measured learning. Content, media and document tools exist, while brand records, editorial workflow and governed distribution are new. Depends on E01–E05, E08, E06 for editorial records, E07 for scheduling, E09/E11 for publishing, and E04-S06 for paid commitments. D03 governs approved workflow policy and exceptions. References: GTM §§6 and 8–11, SK, and FEAS N-2/N-3/N-9.
-A brand owner must be able to maintain approved positioning, proof points, tone and prohibited claims in a versioned, permissioned Messaging Library.
-Content Skills must retrieve approved material. Brand and factual reviews must identify offending passages and supporting evidence, and missing evidence must produce an explicit gap.
-A content operator must be able to create and repurpose articles, landing-page copy, case studies, newsletters, social posts, one-pagers, decks, video scripts and advertising variants for a defined audience and channel.
-Derived assets must retain claim provenance. Documents and media must have previews and linked artifacts, and reusable scripts must avoid repeatedly generating boilerplate.
-An editor must be able to manage a content calendar and review the exact asset intended for publication.
-Brief, draft, review, approved, scheduled, published and failed states must be visible. Reviewer edits must retain version history, and subsequent asset changes must invalidate approval.
-The schedule preview must show channel, account and timezone. Rejected work must return to an assigned owner.
-A marketer must be able to publish approved content to validated channels and verify completion.
-Current account permissions, policy and idempotency must be checked before publication. Provider acceptance must be distinguished from actual publication.
-The final URL, status and metrics must link to the asset. Partial failure across channels must retry only unresolved effects that remain eligible.
-A marketer must be able to run event, community, review and nurture programs with governed follow-up.
-Registrations, invitations, attendance and no-shows, replies, reminders and follow-up must become records or activities and obey consent and stop rules.
-Public-relations statements must receive named approval. Complaints and sensitive community responses must route to an accountable human.
-A paid-marketing owner must be able to plan and optimize advertising within explicit spending limits.
-The preview must show campaign, audience, creative and external advertising budget separately from platform costs.
-Spend-changing actions must follow configured approval bands. Pacing must use reconciled provider actuals and commitments, and missing spending data must stop increases.
-Search optimization, conversion optimization and advertising experiments must distinguish recommendations from changes actually applied.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E15" s="28" t="s">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
         <v>475</v>
       </c>
@@ -16587,32 +17111,11 @@
       <c r="D16" s="26">
         <v>2</v>
       </c>
-      <c r="E16" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — inbound qualification and booking
-Purpose: an inquiry must become an identified, owned opportunity or a correctly routed service request. Voice and gateway components exist, but reliable capture, qualification and booking are new workflows. Depends on E01–E05, E08, E06/E07/E09/E11 and D03's approved workflow and voice-session policy. References: GTM-P4, FEAS N-5, and the GW and VT defects.
-A sales operator must be able to capture inquiries from supported forms, web chat, email, messaging and phone channels.
-Capture must persist the source, time, contact permission and supplied details. Signatures and rate limits must protect intake.
-Repeated submissions must not create duplicate work. Routing must never choose an arbitrary Action or Skill, and unanswered or unroutable inquiries must enter an owned queue.
-A seller must be able to see a new inquiry alongside earlier interactions.
-Identity matching must be explainable and reversible, and account, contact and activity records must retain attribution.
-Existing-customer and support requests must route appropriately. Anonymous or uncertain identities must remain separate until resolved.
-A sales manager must be able to qualify and assign inquiries using explicit business rules.
-Versioned fit and intent scores must show evidence. Assignment must follow capacity, territory and availability rules, with a fallback owner.
-Inactivity must trigger the configured service-level escalation. Model uncertainty must not invent eligibility or a qualification answer.
-A prospect must receive a relevant response using approved product and price facts and permitted history, with an appropriate route to a human.
-Responses must follow the approved workflow or session policy and required exception review. Response-time reporting must distinguish human-review waiting from AI processing.
-Human-escalation requests and opt-outs must be honored.
-A prospect must be able to book a valid meeting in their timezone.
-Availability must be checked before booking, with working hours, buffers, round-robin assignment and attendee timezones applied.
-A last-minute conflict must produce alternatives. Only one provider-confirmed event must be created and linked to the opportunity or activity.
-A prospect or representative must be able to reschedule or cancel and receive appropriate reminders or no-show follow-up.
-Changes must update the same meeting, cancel obsolete reminders and preserve history. Provider failures must be visible.
-Follow-up must use current consent and reply state, and attendance or outcome must close the original booking task.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E16" s="28" t="s">
+        <v>1251</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
         <v>505</v>
       </c>
@@ -16625,32 +17128,11 @@
       <c r="D17" s="26">
         <v>2</v>
       </c>
-      <c r="E17" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — outbound sequences and deliverability
-Purpose: approved outreach must happen at the right time and stop when required. Single-message SMTP and dialer infrastructure exist, while sequences and deliverability controls are new. Depends on the shared E01–E05/E08 foundations, E06/E07/E09/E11, durable approvals and budget controls. A live outbound pilot must wait for those prerequisites. D03 permits routine effects within an approved workflow policy and requires review of exceptions and mandatory checkpoints. References: GTM §§3, 5 and 8–11, and FEAS §3/N-3/N-9.
-An outbound operator must be able to validate a sender and its limits before launch.
-Provider connection, domain authentication and readiness, mailbox identity, daily caps and volume ramp must be visible. Missing setup must block launch.
-Bounce and complaint thresholds must pause affected sending. Rotating mailboxes must not bypass account or domain limits.
-A contact must be able to withdraw permission and have the change enforced immediately.
-Consent must be specific to channel and purpose and retain source, time and evidence. Unsubscribe, complaint, hard-bounce and do-not-call events must update shared suppression.
-Imported lists must not silently clear suppression. Queued steps must check eligibility again immediately before sending or dialing.
-An operator must be able to design, preview and approve a sequence before enrolling contacts.
-Versioned steps must define channel, delay, conditions, template, sending window and exit rules. Previews must show representative recipients, costs and permissions.
-Invalid schedules, loops and missing permissions must fail validation. Active enrollments must retain their selected version until explicitly migrated.
-An operator must be able to trust sequence timing and effects through retries and restarts.
-Deterministic states must determine step eligibility. Each effect must use a stable idempotency key, and leases for each recipient and enrollment must prevent concurrent sends.
-Caps and timezones must apply. Pause, cancellation and uncertain provider outcomes must survive restarts without duplicate contact.
-A seller must be able to take over when a prospect replies or books.
-Replies must link to the correct contact and thread. Replies, bookings and opt-outs must stop or alter enrollment under explicit rules, while ambiguous replies must go to review.
-The next effect must recheck state immediately before dispatch so a recent reply cannot be missed. Handoffs must include qualified context.
-A marketing owner must be able to assess results by cohort and sequence version, including delivery, replies, meetings, failures and suppression.
-Privacy-sensitive open and click tracking must be optional under policy and labelled approximate. Platform cost must be separate from delivery and advertising spend.
-Direct-message and connection automation must remain unavailable unless an approved, supported provider capability exists.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E17" s="28" t="s">
+        <v>1252</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
         <v>535</v>
       </c>
@@ -16663,32 +17145,11 @@
       <c r="D18" s="26">
         <v>2</v>
       </c>
-      <c r="E18" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — deal desk and sales execution
-Purpose: sellers must be able to prepare, qualify, quote and hand off deals using shared evidence. Research and document generation are partly available, while the deal workflow is new. Depends on E06/E09, E05 for grounded answers, E03/E11 for controlled approvals and sends, and E26 for signed contracts, alongside the shared execution, spending and Skill foundations. References: GTM-P6 and GTM §9, FEAS N-2, and BP's sales inventory.
-A seller must be able to prepare a meeting brief and demo plan from verified account context.
-The brief must show stakeholders, interaction history, current needs, open questions and sources. Missing or stale CRM data must be labelled, and interaction history must not be invented.
-A reviewable artifact must be possible from approved uploads before live CRM synchronization is available.
-A seller must be able to turn an authorized recording or notes into confirmed actions and qualification evidence.
-Transcripts and notes must retain provenance and recording permissions. MEDDIC- or BANT-style fields must show evidence and unknowns.
-CRM edits must be proposed as a visible difference from current data. Confirmed actions must have owners and dates, and ingestion of external meetings must remain distinguishable from transcription of platform calls.
-A deal owner must be able to create an accurate quote or proposal within approved terms.
-The Product/Service catalog and Quote and line-item records must support quantity, currency, taxes, validity and versioning. Arithmetic must be deterministic.
-Nonstandard terms and discounts must receive required approval. Approved artifacts must link to the opportunity, and price changes must invalidate affected approvals.
-A presales specialist must be able to draft RFP and security-questionnaire responses from current, accessible, approved evidence.
-Answers must cite sources, assign gaps to experts and respect confidentiality. Claims and certifications must not be invented.
-The final response and attachments must be reviewed before dispatch.
-A manager must be able to inspect deal risks, record quality and forecast changes.
-Missing fields, stale activity, inconsistent stages, competitor and champion signals, and changes in close date must be explainable.
-Updates must follow system-of-record rules. Win and loss reasons must retain evidence, and predictions must remain distinct from confirmed bookings.
-A delivery or customer-success owner must receive an accepted closed-won handoff exactly once.
-Required approvals, signatures and commercial conditions must be verified before accepted scope, obligations, quote and contacts create linked order or onboarding work.
-The recipient must acknowledge ownership. Duplicate close events must not duplicate downstream work, and reopening or cancellation must propagate explicitly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E18" s="28" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
         <v>565</v>
       </c>
@@ -16701,32 +17162,11 @@
       <c r="D19" s="26">
         <v>2</v>
       </c>
-      <c r="E19" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — revenue operations and reporting
-Purpose: owners must be able to trace revenue metrics to business records, interactions and costs. Platform usage reporting exists, while business reporting is new. Depends on E06, the relevant channel, CRM and payment data, and E04's cost ledger, with shared controls and Skills. References: GTM-P2 and GTM §§9–11, and the FEAS §2 correction. A generated research report is not evidence that pipeline reporting already works.
-A revenue owner must be able to inspect funnel, pipeline and conversion by cohort.
-Reports must show lifecycle and stage definitions, period, timezone, currency, deduplication rules and exclusions, with drill-down to records and activities.
-Incomplete or stale synchronization must be visible. Unavailable source data must appear as unknown, never as zero or invented revenue.
-A manager must be able to inspect forecasts and outcomes with explicit assumptions.
-Committed, best-case and forecast figures must be distinguished from won and paid results. Probability versions and missing data must be disclosed and evidence linked.
-Weekly briefs must show risks, required decisions and changed assumptions.
-A marketer must be able to compare channels using a consistent attribution model whose limits are stated.
-First-touch, last-touch and self-reported sources must be available. Conversion windows and identity gaps must be explicit, and multi-touch attribution must not be presented as proof of causation.
-Campaign, content and sequence lineage must survive record merges and CRM synchronization.
-An owner must be able to inspect cost per qualified opportunity, meeting and sale.
-Platform, provider and campaign costs must reconcile to their ledgers and the relevant outcome cohort.
-Cancelled, duplicate and failed activities must be treated consistently. Missing external spend must be disclosed, and margin and return-on-investment calculations must show assumptions.
-An owner must be able to see what the AI workforce did and what needs attention through an activity feed filtered by business object, workflow and outcome.
-The feed must link runs, costs, approvals and artifacts, including failures, skipped actions and waiting work.
-The business result must be understandable without reading raw internal traces.
-A revenue-operations owner must be able to turn performance findings into controlled improvement proposals.
-Alerts must use configured thresholds and data freshness. Proposals must identify affected Skills or rules and their evidence, while human edits and rejections must feed evaluation.
-A recommendation must not silently change pricing, outreach or policy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E19" s="28" t="s">
+        <v>1254</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
         <v>595</v>
       </c>
@@ -16739,32 +17179,11 @@
       <c r="D20" s="26">
         <v>2</v>
       </c>
-      <c r="E20" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — customer care, retention, and expansion
-Purpose: customers must receive continuous, accountable help from onboarding through renewal. Channel and knowledge-base components exist, while customer operations are new. Depends on E05/E06/E07/E09/E11/E18 and the shared platform controls. This is an H4 module, supporting local records and declared external masters. It adds Ticket, Customer Onboarding Plan, Service Entitlement, Health Snapshot and Renewal records, reusing Account, Contact, Activity and Opportunity. References: GTM §9's lifecycle signals and BP's support, retention and education inventory.
-A customer must be able to report a problem across supported channels and receive an accountable response.
-Intake must create or deduplicate a ticket, determine entitlement and priority, assign an owner and response deadline, and link related conversations.
-Urgent and security cases must route to the appropriate incident owner. Closure must record a resolution or an explicit unresolved state.
-A support operator must be able to resolve known issues from approved evidence and escalate the rest.
-Suggested answers must cite current knowledge and product context. Diagnostic tools must use scoped permissions.
-Low confidence, failed remediation and requests for a human must trigger handoff with history. Customer responses must follow communication policy, and feedback may propose a knowledge-base update for review.
-A customer-success owner must be able to turn the accepted sales promise into an onboarding plan.
-The plan must include customer goals, commitments, tasks, owners, dates and acceptance conditions. Completion must be supported by evidence, blocked tasks must escalate, and scope changes must require an explicit decision.
-Customer appointments must reuse the existing booking capability.
-A customer must be able to obtain relevant training and approved self-service material.
-Guides and tutorials must be versioned and linked to the applicable product and entitlement. Completion and unresolved questions must be recorded.
-Repeated questions must be able to propose content improvements. Inaccessible or obsolete material must not be presented as current guidance.
-An account owner must be able to identify customers at risk or ready for expansion and act on the evidence.
-Health must combine declared usage, support and payment inputs with freshness and explainable weights. Risks must create assigned interventions, and renewal dates must trigger governed tasks.
-New commercial terms must use quote and contract approval rather than silent account changes.
-An account owner must be able to prepare quarterly business reviews, feedback surveys and advocacy requests.
-Review metrics must link to records, and surveys and review requests must obey consent and contact policy.
-Complaints must route to service recovery. Case studies and public references must have customer permission, and participation must be measured separately from satisfaction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E20" s="28" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
         <v>627</v>
       </c>
@@ -16777,27 +17196,11 @@
       <c r="D21" s="26">
         <v>2</v>
       </c>
-      <c r="E21" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — orders, delivery, and fulfillment
-Purpose: an accepted commercial promise must become a tracked, delivered and accepted product or service. This is a new H4 business module using shared records, events, Skills, integration ownership and platform controls. Depends on E06/E07/E17/E26, E22 for purchased inputs and E21 for billing. It adds Order/Line, Project, Task, Milestone, Deliverable, Acceptance, Shipment and Return records and reuses the Product/Service catalog. References: GTM's closed-won handoff and BP's delivery inventory.
-A delivery manager must be able to plan accepted work against capacity and dependencies.
-Approved scope must create one linked order or project. Tasks must identify owners, required resources, dependencies and deadlines, and overcommitment must be visible.
-Scope changes must preserve the original commitment and obtain required approval.
-A customer or authorized reviewer must be able to inspect a deliverable, accept it or request rework.
-Completion must require the specified evidence and reviewer authority. Quality checks and proof of work must remain linked to the deliverable.
-Partial acceptance and rework must remain visible. An accepted milestone must emit only one eligible billing or handoff event.
-An operations owner must be able to fulfill stocked goods or provision a service without promising unavailable capacity.
-Inventory or resource availability must be checked and reserved before confirmation. Shipment and provisioning status must come from actual execution or provider evidence.
-Failures must create owned exceptions. Detailed production and bill-of-materials planning must remain an optional, separately scoped capability.
-A service operator must be able to manage delays, returns and corrective action.
-Service-level risks must alert the accountable owner, and customer communications must receive required review.
-Returns must track eligibility, receipt, inspection and disposition. Refunds must use the authorized finance workflow.
-Order, project and inventory state must reconcile after cancellation or retry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E21" s="28" t="s">
+        <v>1256</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="27" t="s">
         <v>650</v>
       </c>
@@ -16810,26 +17213,11 @@
       <c r="D22" s="26">
         <v>2</v>
       </c>
-      <c r="E22" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — invoicing and collections
-Purpose: accepted commercial obligations must become correct invoices, receipts and reconciled balances. This is a new H4 business-finance module, separate from HireBuddha's platform billing. Depends on E04's external-commitment controls, E06/E07/E09/E11/E17, E23 for accounting and the shared approval and execution services. It adds Invoice/Line, Receivable, Receipt, Credit Note and Collection Case records and reuses Order, Contract and Payment. References: BP's receivables inventory, RT's HBS concept and the GTM payment-attribution extension.
-A finance operator must be able to issue a reviewed invoice from accepted terms or delivered milestones.
-Amounts, taxes, currency, numbering, due date and billing party must be validated. Draft, issued, void and credited states must be explicit.
-Issued history must remain immutable and be corrected through adjustments. Repeated milestone events must not produce duplicate invoices.
-A finance operator must be able to record and allocate payments accurately.
-Provider callbacks and imports must have their source verified and be deduplicated. Partial payments, overpayments, underpayments and fees must be explicit.
-Receipt allocations must reconcile to outstanding invoice amounts. Failed or reversed settlement must reopen the appropriate balance while retaining history.
-An accounts-receivable owner must be able to follow up on overdue balances with the correct context and contact limits.
-Deterministic reminders must use the current outstanding balance, agreed time windows and contact policy.
-Disputes, confirmed payment and manual holds must stop inappropriate reminders. Collection actions and promises to pay must have recorded owners and dates.
-A finance reviewer must be able to resolve a dispute or approve a credit, refund or write-off.
-The review must include contract, delivery and support evidence and show financial impact. Required independent and authorized approval must apply.
-The adjustment must update receivables and accounting exactly once. The customer must receive only the approved outcome, and the complete case must remain auditable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E22" s="28" t="s">
+        <v>1257</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="27" t="s">
         <v>673</v>
       </c>
@@ -16842,27 +17230,11 @@
       <c r="D23" s="26">
         <v>2</v>
       </c>
-      <c r="E23" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — procurement and payables
-Purpose: goods and services must be purchased, and suppliers paid, under controlled authority. This is a new H4 module using the shared platform services and declared system-of-record ownership. Depends on E03/E04/E06/E07/E09/E23/E26. It adds Vendor Profile, Requisition, Purchase Order, Goods/Service Receipt, Supplier Bill, Payment Instruction and Verification Result records. References: BP's procurement, vendor and payables inventory, and RT's ownership and separation-of-duties requirements.
-A procurement owner must be able to assess suppliers and activate an approved vendor.
-Vendor identity, risk, insurance and compliance documents, and verification freshness must be recorded. Adverse findings must escalate.
-Bank-detail changes must receive independent verification. The person who creates a vendor must not authorize its payment.
-A requester must be able to obtain an approved purchase for a documented business need.
-The requisition must compare available suppliers, terms and budget. Approval must create a versioned purchase order.
-Changes and cancellations must update commitments, and the requester must be able to see delivery or service acceptance and any exceptions.
-An accounts-payable operator must be able to match a bill to authorized purchasing and receipt evidence.
-Duplicate-invoice checks and checks of amounts, quantities, taxes and purchase-order or receipt tolerances must be deterministic.
-Unmatched differences must create an owned exception. Matching a bill must not itself authorize payment.
-An authorized payer must be able to execute a reviewed payout and know the settlement outcome.
-Beneficiary, bank-detail version, amount, currency, due date, authority and funds must be rechecked before payment.
-Maker/checker separation and dual-approval rules must apply. Stable idempotency and provider reconciliation must prevent duplicate payouts.
-Pending, failed and reversed transactions must remain distinguishable from paid transactions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E23" s="28" t="s">
+        <v>1258</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
         <v>696</v>
       </c>
@@ -16875,27 +17247,11 @@
       <c r="D24" s="26">
         <v>2</v>
       </c>
-      <c r="E24" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — accounting and financial close
-Purpose: tenants must be able to maintain consistent business books with traceable evidence. This is a new H4 module; platform usage logs do not constitute business accounts. Depends on E06/E09, transactional feeds from E21/E22, E03 review and the shared platform services. It adds Chart of Accounts, Journal/Entry/Line, Accounting Period, Bank Statement/Line, Reconciliation, Expense Claim and Tax Code records. References: BP's accounting, expenses and tax inventory, and RT's HBS concept. Supported local scope and externally mastered accounting must be declared explicitly.
-An accountant must be able to post balanced, evidence-backed transactions and correct them visibly.
-Deterministic double-entry checks must prevent imbalanced entries. Currency, posting date and account must be validated.
-Posted entries must be immutable, with corrections recorded as reversals or adjustments. Open and closed accounting periods must be enforced.
-Source documents and approved business events must link to the entries they support.
-A bookkeeper must be able to reconcile bank and payment records and employee expenses.
-Imports must be deduplicated and retain their source. Suggested matches must show evidence and confidence, and approved matches must be distinguished from unmatched exceptions.
-Expense claims must include receipts, policy checks and review. Adjustments must not bypass accounting controls.
-A finance owner must be able to close a period and produce reconciled management accounts.
-The close checklist must cover unresolved matches, receivables, payables and required adjustments. The trial balance and supported statements must reconcile to journal entries.
-Reopening a period must require authority. Missing inputs must prevent a claim that the close is complete without exceptions.
-A domain reviewer must be able to configure supported taxes and prepare required financial reports.
-Tax and jurisdiction rules must be versioned with sources and effective dates. Arithmetic must follow deterministic rules or approved providers.
-Unsupported requirements must be explicit. Filings and statutory submissions must receive qualified review and approval, and the product must not claim universal global compliance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E24" s="28" t="s">
+        <v>1259</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="27" t="s">
         <v>719</v>
       </c>
@@ -16908,26 +17264,11 @@
       <c r="D25" s="26">
         <v>2</v>
       </c>
-      <c r="E25" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — planning, treasury, and forecasts
-Purpose: leaders must be able to decide budgets and cash actions from stated assumptions and actual business data. This is a new H4 module using shared controls, records, events, Skills and integration ownership. Depends on E06/E18/E21–E23. It adds Business Budget, Budget Version, Cash Forecast, Scenario, Target and Variance records, separate from platform-spending envelopes. References: the GTM reporting extension and BP's planning, pricing and treasury inventory.
-An owner must be able to set operating targets and approve departmental budgets.
-Budget versions must identify period, currency, assumptions, owner and approval. Actuals and commitments must reconcile to business ledgers.
-Variance alerts must use configured thresholds. Changes must retain history and must not automatically change the AI wallet.
-A treasury owner must be able to inspect cash balances, expected receipts and payments, and runway.
-Forecasts must distinguish cleared, committed, expected and speculative cash and show timing assumptions, foreign-exchange assumptions and stale feeds.
-Scenarios must allow collection, hiring and spending assumptions to change. Any movement of cash must remain a separately approved action.
-A finance leader must be able to compare reproducible forecast scenarios and record a decision.
-Scenarios must use versioned inputs, expose assumptions and sensitivities, and support recommendations with evidence.
-Approval must create owned follow-up work rather than silently reallocating funds.
-An owner must be able to receive a management pack combining financial and operational results.
-Each metric must identify its period, currency, source and freshness and allow drill-down. Narrative must distinguish observed facts from inference.
-Risks and decisions must have owners. Restricted financial information must retain its access controls in Pragya and in exports.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E25" s="28" t="s">
+        <v>1260</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="27" t="s">
         <v>741</v>
       </c>
@@ -16940,32 +17281,11 @@
       <c r="D26" s="26">
         <v>2</v>
       </c>
-      <c r="E26" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — people lifecycle
-Purpose: recruiting, employment operations and exits must remain coordinated and accountable to humans. This is a new H4 domain reusing generic document and channel capabilities and shared platform services. Depends on E01/E03/E05/E06/E07/E09/E11/E26/E28. It adds Position, Requisition, Candidate, Application, Interview, Employee, Employment Agreement, Leave, Payroll Input, Review, Training and Exit Case records. References: BP's people, recruiting, payroll, benefits and training inventory. Full local payroll requires separately validated jurisdiction scope.
-A recruiter must be able to coordinate sourcing, applications, interviews and evidence-based screening.
-Job criteria and screening rubrics must be approved and versioned. Candidate consent and data scope must be recorded.
-Evaluations must cite job-related evidence and uncertainty. Human reviewers must own consequential hiring decisions, while scheduling and communications must reuse governed capabilities.
-A hiring manager must be able to prepare an offer within an approved role and compensation range.
-The requisition, compensation and terms must be checked. Every offer and nonstandard negotiation must receive the assigned human's approval.
-The final agreement must be versioned and signed through E26. Declined or expired offers must not trigger onboarding.
-An employee must be able to complete onboarding, request leave and receive policy answers.
-The employee record must control scoped access. Onboarding tasks must have owners and completion evidence, and leave balances and approvals must follow deterministic rules.
-Answers must cite the applicable policy. HR cases must remain private and escalate when uncertain.
-A payroll or people operator must be able to prepare reviewed payroll inputs and development records.
-Approved hours, leave, compensation changes and reimbursements must reconcile to their sources, with exceptions sent for review.
-Payroll output must target an approved provider or a separately validated local jurisdiction module. Training and appraisals must use transparent criteria and human review.
-An HR owner must be able to execute an approved exit with coordinated access and asset handling.
-The separation decision must be human-authorized. Revocations, asset return, knowledge handover and final-pay inputs must have owners and effective dates.
-Failed or delayed revocation must escalate. Statutory requirements and legal holds must be checked, and completion must be based on evidence.
-An authorized people leader must be able to inspect workforce needs and trends without exposing private records.
-Headcount, capacity, leave and training metrics must obey access and aggregation rules. Predictions must be labelled and must not automatically cause adverse employment action.
-Record corrections and approved exports must be supported.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E26" s="28" t="s">
+        <v>1261</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="27" t="s">
         <v>772</v>
       </c>
@@ -16978,27 +17298,11 @@
       <c r="D27" s="26">
         <v>2</v>
       </c>
-      <c r="E27" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — contracts and obligations
-Purpose: legal and commercial work must move from a request to approved terms, verified signature and tracked obligations. Document generation exists, while contract lifecycle management is a new H4 module. Depends on E03/E05/E06/E09/E11 and shared scheduling, execution and Skill services. It adds Contract, Contract Version, Clause/Playbook, Approval, Signature Envelope, Obligation and Dispute records. References: GTM's proposals and redlines, and BP's legal inventory.
-A contract owner must be able to draft from approved templates and inspect deviations.
-Variables must link to verified business records, and the template and playbook versions must be pinned.
-Comparison and redlines must reveal changed terms and missing information. Liability and nonstandard terms must go to qualified human review.
-An unreviewed legal conclusion must not become an approved clause.
-A legal reviewer must be able to authorize the exact version and signing parties.
-Review must cover commercial authority and exceptions. Edits must invalidate prior approvals where appropriate, and signatory identity and authority must be checked.
-Rejected or outdated versions must not be sent for signature.
-A contract owner must be able to route an approved agreement and verify its execution.
-Creating an e-signature envelope must be idempotent. Signed, declined, expired and provider-pending states must be verified rather than inferred.
-The executed document and signature evidence must be stored. Only verified execution must trigger downstream commitments.
-An obligation owner must be able to monitor renewals, notice dates, duties and disputes.
-Extracted obligations must be reviewable and linked to their clauses. Reminders must have owners and due dates.
-Changes and termination must preserve contract history. Disputes must link relevant support, delivery and finance evidence, and deadlines must not silently lapse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E27" s="28" t="s">
+        <v>1262</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="27" t="s">
         <v>795</v>
       </c>
@@ -17011,32 +17315,11 @@
       <c r="D28" s="26">
         <v>2</v>
       </c>
-      <c r="E28" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — risk, privacy, and incidents
-Purpose: business obligations, privacy requests and incidents must reach accountable people with reliable evidence. Some platform controls exist, while these H4 business workflows are new. Depends on E01/E03/E05/E06/E07/E09/E12 and independent audit permissions, using shared Skills and controls. It adds Risk, Control, Policy/Obligation, Evidence, Privacy Request, Legal Hold, Incident, Action and License/Insurance Record families. References: GTM's compliance and privacy requirements and BP's risk, incident and corporate-record inventory.
-A risk owner must be able to maintain applicable obligations and an owned control plan.
-Applicability must be reviewed for the supported jurisdiction and sector, including required sustainability or ESG disclosures.
-Each obligation must record source, effective date, owner, evidence and due date. Changes must create reviewed tasks, and monitoring must not imply universal legal compliance.
-An independent auditor must be able to sample controls and track findings.
-Evidence must retain provenance, time, integrity checks, scoped retention and access history. Auditors must not alter the operations they audit.
-Findings must have severity, owner and remediation evidence. Corporate licenses and insurance renewals must receive owned reminders.
-A privacy officer must be able to fulfill a verified person's access, correction or deletion request.
-Identity and request scope must be verified, and relevant business records, conversations, knowledge and derived stores must be enumerated.
-Legal holds must be detected and a reviewer must authorize the actions. Fulfillment must record completion and exceptions and notify downstream systems according to declared responsibility.
-A data owner must be able to understand and govern where business data is used.
-The data map must cover integrations, models, logs, artifacts and backups, with explicit retention, residency and training choices.
-Operational processing consent must not imply model-training consent. Revoked or deleted data must not be silently reused by new learning jobs.
-An incident commander must be able to receive reports from any permitted source and triage, contain and recover a business or security incident.
-Severity, owner, runbook and timeline must be recorded. Safe pre-authorized containment must be deterministic and bounded, and unsafe work must be stoppable promptly.
-Recovery must require evidence and controlled re-enablement.
-An accountable leader must be able to review customer, public and regulatory incident communications and learn from the event.
-Drafts must identify verified facts and uncertainty. Named humans must authorize required communications, and deadlines and delivery outcomes must be tracked.
-Postmortems must assign corrective actions. Deterministic incident status and notifications must remain available when the funded AI reserve is exhausted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E28" s="28" t="s">
+        <v>1263</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="27" t="s">
         <v>826</v>
       </c>
@@ -17049,26 +17332,11 @@
       <c r="D29" s="26">
         <v>1</v>
       </c>
-      <c r="E29" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — access, assets, and operational maintenance
-Purpose: people and workflows must have the right systems and assets, with predictable maintenance. Some technical tools exist, while business administration is a new H4 module using shared platform services. Depends on E01/E03/E06/E07/E09/E12/E25. It adds Access Request/Grant, Asset, Assignment, Maintenance Plan, Service Ticket and Data Job records. References: BP's IT, facilities and data-pipeline inventory, and GTM's connector-health requirements.
-An IT owner must be able to provision and revoke approved access using least privilege.
-Requests must link to a verified person or role and an approval. Privileged access must receive independent review.
-The target system must confirm granted scopes and effective dates. Failures must remain open, and recertification and exit revocation must retain evidence.
-An operations administrator must be able to track physical and digital assets and recurring maintenance.
-Records must show ownership, assignment, lifecycle, licenses or leases and renewal dates. Planned work must have owners and due dates.
-Overdue maintenance and unused licenses must raise proposals. Purchases and disposals must follow procurement and approval policy.
-A data owner must be able to identify and repair stale or failed business-data flows.
-Freshness and quality checks must link to the relevant jobs and records. Schema changes and reconciliation gaps must create owned exceptions.
-A repair preview must preserve system-of-record rules and idempotency, and reconciliation after repair must demonstrate consistent data.
-A service owner must be able to restore an integration using an approved runbook or a reviewed fix.
-Diagnosis must collect evidence without exposing secrets. Known low-risk runbooks must respect permissions and limits.
-Generated code and adapter changes must enter E32's independent testing and promotion process. Failed repair must escalate instead of repeatedly changing production.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E29" s="28" t="s">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="27" t="s">
         <v>849</v>
       </c>
@@ -17081,26 +17349,11 @@
       <c r="D30" s="26">
         <v>1</v>
       </c>
-      <c r="E30" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — product, experiments, and pricing
-Purpose: the business must turn customer and market evidence into considered product and offer changes. This is a new H4 workflow using shared records, events, Skills, integration ownership and controls. Depends on E06/E13/E18/E19/E24 and E03 for commercial or publishing changes. It adds Idea, Research Finding, Product Requirement, Backlog Item, Experiment, Offer/Price Version and Launch Plan records. References: GTM's voice-of-customer, conversion-optimization and competitive research needs, and BP's product and pricing inventory.
-A product owner must be able to synthesize customer, market and support evidence into a prioritized backlog.
-Findings must preserve source, permission and affected segment. Duplicate requests must consolidate without losing their counts.
-Prioritization must expose impact, effort and uncertainty assumptions. Humans must approve commitments, and customer statements must not become fabricated roadmap promises.
-A launch owner must be able to coordinate an approved product or service release.
-Scope, acceptance, enablement, support readiness, fulfillment and marketing work must have owners. Launch must depend on actual readiness evidence.
-Content and price publication must obey approvals, and rollback and handling of customer impact must be defined.
-An experiment owner must be able to test a hypothesis with agreed measurement and stop rules.
-Population, allocation, success measures, guardrail measures, duration and consent constraints must be explicit.
-Data gaps must be visible, and early stopping and exclusions must be documented. Analysis must not claim causation from unqualified correlations.
-A commercial owner must be able to compare pricing and packaging proposals before applying them.
-Proposals must use cost, demand and contract constraints, with audience, percentage and amount limits and required approval.
-Contractual prices must remain protected. Activated price versions must propagate consistently to quoting and billing and support audited reversal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E30" s="28" t="s">
+        <v>1265</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="27" t="s">
         <v>871</v>
       </c>
@@ -17113,32 +17366,11 @@
       <c r="D31" s="26">
         <v>1</v>
       </c>
-      <c r="E31" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — partnerships and capital stakeholders
-Purpose: partner, board, investor and corporate-development work must share business evidence under explicit authority. This is a new H4 module reusing research, documents and shared platform services. Depends on E06/E09/E13/E17/E18/E24/E26/E27. It adds Partner Profile, Partner Agreement, Referral, Commission, Stakeholder, Board Action, Diligence Request and Data Room records and reuses Account and Contact. References: GTM's later partner and channel backlog and BP's partnerships and capital inventory.
-A partnership owner must be able to evaluate and onboard a business partner.
-Due diligence, territory, rights, enablement and agreement terms must be recorded, and required review must finish before activation.
-Partner access must expose only shared records. Channel-enablement content must be current and approved.
-A channel manager must be able to track referrals, co-selling and earned commission.
-Referral ownership, deduplication and attribution rules must be explicit. Deal and receipt state must determine eligibility, and disputes must go to review.
-Commissions must reconcile to approved agreements, and payouts must use E22's controls.
-A leader must be able to prepare board and investor reports and retain the decisions that follow.
-Reports must use permissioned, reconciled business metrics and disclose narrative assumptions. External sends must receive named review.
-Meetings must create accepted actions with owners and dates, and confidential strategy must remain separately scoped.
-A capital-process owner must be able to maintain an access-controlled diligence room and research funding or acquisition opportunities.
-Documents must have versions, purpose-limited access and expiry. Requests and answers must have owners, and access and downloads must be audited.
-Research must cite sources. Negotiation and financial commitments must require explicit human authority.
-An executive must be able to delegate scheduling, inbox triage and meeting preparation within explicit boundaries.
-Internal communications must be classified with scoped access. Proposed replies and meetings must use approved channel and calendar controls.
-Conflicts and sensitive requests must route to the owner. Minutes must cite source notes and produce confirmed action items without inventing commitments.
-An owner must be able to turn strategic decisions into owned work and review progress.
-Objectives must link to initiatives, budgets, measurable outcomes and accountable people. Changes must retain the decision rationale.
-Periodic reviews must show actual progress, blockers and assumptions. Cross-functional assignments must require acceptance and must not silently override another owner's authority.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E31" s="28" t="s">
+        <v>1266</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="27" t="s">
         <v>902</v>
       </c>
@@ -17151,38 +17383,11 @@
       <c r="D32" s="26">
         <v>1</v>
       </c>
-      <c r="E32" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — model routing and multimodal work
-Purpose: operators must be able to choose an eligible model or use evaluated automatic selection while retaining quality, policy and cost controls. Vendor adapters and static defaults exist, while dynamic routing and unified asynchronous media jobs are new. Depends on E01/E02/E04/E05/E08/E12 and E32 for learned preferences. D29 defines the required provider catalog, with exact versions and capabilities to be validated during implementation. References: RF §3, §6.4 and §8, RT §§3–5, and the LP and TL defects.
-An administrator must be able to restrict models by capability and data policy.
-The registry must show supported modalities, context limits, tools and approved usage policy. Tenant constraints must filter candidates before selection.
-Pinning an unavailable or ineligible model must cause an explicit failure or a configured eligible fallback. Fallback must never bypass data restrictions.
-An owner must be able to choose Auto and understand its quality and cost tradeoff.
-Routing must consider task class, modality, context, latency, cost ceiling and measured performance, and record the decision and actual cost.
-If no eligible model exists, work must visibly block or enter a declared degraded state. Automatic routing must be tested against the static incumbent before production use.
-An operator must be able to recover from provider failures without repeating business effects.
-Bounded timeouts and retries must distinguish generation from tools that already executed. Fallback must retain context without repeating confirmed effects.
-Cancellation must settle known usage. Provider failures and incompatible tool schemas must produce actionable outcomes.
-A content author must be able to request image, video, editing or audio work and follow progress without blocking other work.
-Jobs must show queued, running, completed, failed and cancelled states, with previews, artifacts and attributed cost. Asynchronous completion must be verified with the provider.
-Unsupported options must fail clearly. Retries must not accidentally charge for or publish duplicate outputs.
-A quality owner must be able to admit or retire models using independent task cohorts.
-Evaluation must measure quality, tool and schema accuracy, cost, latency and policy compliance. Changed model versions must have regression evidence, rollback and reporting of affected workflows.
-Benchmark scores alone must not enable production use.
-A voice or media owner must be able to select a provider validated against the actual language, interruption, tool, latency and artifact requirements of a supported use case.
-Quality thresholds must be agreed per use case. Mid-call failure must follow a tested transfer or closure plan, and every new provider must pass capability-specific acceptance.
-An administrator must be able to enable validated adapters and capability profiles for Gemini, Claude, OpenAI, GLM, Qwen and Kimi.
-Credentials must be tenant-scoped. Model and version, region, modality and data-policy constraints must be explicit, and unavailable providers must fail clearly rather than being implicitly selectable.
-A content owner must be able to use the supported video capabilities for Veo, Seedance and Wan, with asynchronous status, cancellation, policy checks, usage attribution, persistent artifacts and duplicate-publication protection.
-The supported image catalog must include Gemini Image, GPT Image, Qwen Image and Kling with capability-specific options, safety checks, previews, artifacts, cost attribution and deterministic failure handling.
-Unsupported image-option combinations must be rejected before spending.
-A platform owner must be able to replace or add a model without rewriting business workflows.
-Adapters must implement a common contract. Version pinning, fallback eligibility, routing decisions, migration and rollback must all be recorded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E32" s="28" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="27" t="s">
         <v>949</v>
       </c>
@@ -17195,32 +17400,11 @@
       <c r="D33" s="26">
         <v>4</v>
       </c>
-      <c r="E33" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — evaluated learning and self-improvement
-Purpose: improvements must earn deployment through evidence and remain reversible. Memory, reflection and Board machinery partly exist with integration defects, while the complete promotion cycle is new. Depends on E02–E05, E08, E12 and relevant business metrics. Decisions D15 and D23 require independent evaluation and authorized promotion rather than self-approval or calendar-based improvement claims. References: SK §11, GTM §11, RF §§5, 10 and 12, RT §§7, 9 and 22, and the MI, MC and PC defects.
-A quality owner must be able to link human feedback and business outcomes to the versions that produced them.
-Run, Skill, model and policy versions must link to success, edits, rejections, complaints, cost and delayed outcomes. Missing labels must remain unknown.
-Feedback must obey consent and access restrictions, and metrics must support comparisons between equivalent cohorts.
-A workflow owner must be able to assess a candidate before replacing the incumbent.
-Independent curated cases and reference cases from the incumbent must include negative and adversarial scenarios. Skipped tests or exhausted test budgets must not count as passes.
-Human spot checks must supplement automated scoring. The report must show regressions and changes in cost and latency.
-A capability owner must be able to turn repeated successful work into a reusable Skill proposal.
-The proposal must link observed patterns and examples, define scope and proposed scripts or instructions, and check for existing reusable work before creating a duplicate.
-The candidate must pass E08's authoring requirements and E32's evaluation and remain inactive until promotion is authorized.
-A workforce owner must be able to test and adopt improved instructions or routing preferences.
-The proposal must state evidence and expected benefit. An approved limited rollout must compare the candidate with the incumbent under bounded exposure.
-Predefined regression rules must automatically restrict or roll back the change. Original versions and decisions must remain auditable, and improvement must not be guaranteed merely because time has passed.
-A service owner must be able to request a missing or repaired capability without allowing unreviewed changes to live behavior.
-Generated code must execute only in the approved isolated runtime and undergo independent tests, permission checks, metering and adversarial checks.
-Ordinary tenant Skills must not rewrite sensitive primitives. The exact changes and their impact must be presented for independent human approval.
-An operator must be able to promote or roll back a reviewed capability safely.
-The promoter must be distinct from the author or proposer. The active-version change must be atomic, distributed workers must converge on it, and handling of in-flight runs pinned to prior versions must be explicit.
-A failed limited rollout must disable affected effects and restore a known version. Since rollback cannot undo real-world effects, it must create reconciliation tasks where required.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E33" s="28" t="s">
+        <v>1268</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="27" t="s">
         <v>979</v>
       </c>
@@ -17233,29 +17417,11 @@
       <c r="D34" s="26">
         <v>3</v>
       </c>
-      <c r="E34" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — Generative and adaptive experience
-Purpose: a new frontend must help people operate their business through appropriate conversational and structured views. This is new work, while the current frontend must remain usable in earlier releases. Depends on the supported capabilities' APIs and authorization, E10's Pragya flow and E06's schema metadata. D05 requires an explicit Design Gate before implementation, D26 makes Pragya the single human workspace, and D31 requires the digital-twin experience developed with E39/E40. References: RF §11, RT §8 and the confirmed product decisions.
-A product owner must be able to approve a complete experience direction before frontend development starts.
-Design and brainstorming must cover owner, operator, reviewer and administrator journeys, information architecture, interaction prototypes, visual language, accessibility, mobile behavior and failure states.
-Review must test realistic work and record decisions. Implementation of the new frontend must wait for explicit design acceptance.
-A reviewer or operator must be able to understand how generated views retain user control.
-Prototypes must demonstrate record detail and editing, activity feeds, approvals, budgets, workflow configuration and handoff to Pragya.
-Consequential actions must have stable, discoverable controls. Unsupported generation must have a usable fallback, and research must measure comprehension as well as appearance.
-A user must be able to receive a task-appropriate view and retain a preferred arrangement.
-Generated view definitions must select approved components and validated data bindings. Backend authorization must govern every data and action request.
-Generated views must not introduce arbitrary executable UI code or grant additional access. Preferences must be editable and resettable, and stale or incompatible schemas must produce a useful recovery state.
-An existing user must be able to move to the new frontend without losing essential workflows.
-The parity checklist must include authentication, records, execution, artifacts, approvals, integrations, budgets and account administration.
-Migration must be staged, monitored and reversible. The current UI must remain available until its replacements pass, and accessibility and task success must be measured.
-The Pragya workspace must support voice-first interaction alongside text, direct visual edits, analytics drill-down and immediate stop.
-The experience must include a detailed isometric 3D digital twin and a knowledge and assets explorer. It must show available levels first, with a usable accessible alternative.
-Persisting all six organizational levels must depend on the optional E40 Graph/Loop capability rather than inventing a mandatory legacy hierarchy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E34" s="28" t="s">
+        <v>1269</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="27" t="s">
         <v>1001</v>
       </c>
@@ -17268,27 +17434,11 @@
       <c r="D35" s="26">
         <v>2</v>
       </c>
-      <c r="E35" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — product packaging and organizational scale
-Purpose: a business must be able to adopt useful workflows progressively and expand its organizational scope safely. Tenant and partner hierarchy exist, while modular packaging and business-unit governance are new. Depends on E01/E04/E06/E09/E12 and the capabilities included in each package. D01 rejects inherited bundle and agent counts, while D32 supports ad hoc work alongside Solo, MSME, startup and enterprise package candidates whose contents and prices remain open. References: GTM's tenant-zero and commercial questions, useful adoption and scale needs from BP, and the product decisions.
-A buyer must be able to understand the outcomes a package supports and the prerequisites it needs.
-Each package must identify supported workflows, integrations, required human roles, autonomy, limitations and usage estimates.
-A fixed agent count must not be the value promise. Activation must check prerequisites and create only the needed configurations, and failed setup must remain recoverable.
-A commercial owner must be able to price and support a package using measured economics.
-Tenant-zero evidence must include actual workloads, outcomes, variable costs, idle storage costs, reviewer effort and support burden.
-The commercial model and free allowance must be explicitly chosen under O04. Unapproved per-seat or per-outcome prices must not be treated as settled decisions.
-Plan changes must preserve entitlements and records. A finite ad hoc task must not require activation of an entire business package.
-A group owner must be able to manage business units with different budgets, policies and data access.
-Parent visibility must be explicit. Approved policies must inherit downward and metrics aggregate upward, with no default sharing between siblings.
-Storage and processing placement must actually satisfy model and residency requirements. Separate legal entities and currencies must not be combined into misleading totals.
-A partner administrator must be able to support assigned businesses within their boundaries.
-Assignments and delegated roles must determine access. Pricing and branding privileges must be bounded, and support actions must identify the actor in the audit trail and use time-limited access where appropriate.
-Tenant offboarding must revoke delegation and preserve the tenant's export rights.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E35" s="28" t="s">
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="27" t="s">
         <v>1025</v>
       </c>
@@ -17301,26 +17451,11 @@
       <c r="D36" s="26">
         <v>4</v>
       </c>
-      <c r="E36" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — BabyBuddha and OmniBuddha research
-Purpose: in-house models may be used if comparative evidence shows better task quality or lower cost. This is a research aspiration, not a shipped capability, an approved investment or a prerequisite for the business product. Depends on E31/E32 and explicit permission to use data. H6 is an investment decision rather than a promised launch. References: RF §3.1 and §8.1, and RT §§3 and 5.
-A data owner must be able to choose whether eligible traces can be used in model development.
-Explicit opt-in must record the permitted purpose and data categories. Tenant-secret and personal-data restrictions must apply, and withdrawal must stop future collection within that scope.
-Data lineage and retention must be reviewable. Operational memory must not be treated as implied training consent.
-A research sponsor must be able to decide whether post-training an open-weight model is worthwhile.
-The research proposal must document licensing and serving constraints, the approved dataset, incumbent baselines, task cohorts and full cost.
-Evaluation must compare tool use and reasoning, or multilingual speech quality, as appropriate. Evidence must determine whether research continues or stops.
-A model owner must be able to propose BabyBuddha for eligible text and tool workloads.
-Fast and reasoning profiles must pass independent quality, safety, tool-reliability, latency and cost checks against the incumbent.
-A limited rollout and eligible fallback must exist. Without sufficient evidence, current providers must remain the default.
-A voice owner must be able to propose OmniBuddha for a validated speech workload.
-Tests must cover supported languages, switching languages within a conversation, interruption, tool calls, consent handling, latency and funded safe closure.
-Failed calls must have tested handoff or termination behavior. Production admission and rollback must use E31/E32's controls.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E36" s="28" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="27" t="s">
         <v>1047</v>
       </c>
@@ -17333,32 +17468,11 @@
       <c r="D37" s="26">
         <v>1</v>
       </c>
-      <c r="E37" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — isolated relational tenant data plane
-Purpose: every tenant must have a queryable, exportable relational business database, and no tenant may access another tenant's business payload. Shared models and operational tables exist, but the isolated relational data plane is new. Depends on E01/E02/E03/E04/E06/E07/E09/E12. Decisions D02, D09 and D25 confirm typed relational storage and the shared-control-plane boundary. References: the tenant and ad hoc backlog, the operating model and product decisions.
-A tenant must be able to store business records in a dedicated relational database.
-The database must use typed tables, foreign keys, constraints, indexes and reviewed versioned migrations.
-Campaigns, contacts, activities, finance and other module records must be queryable without a generic JSONB record store or JSONB custom-field bag.
-A Skill or application must be able to use a safe tenant data API.
-Every request must be tenant-scoped and authorized. Filtering, sorting, pagination, transactions, validation, optimistic concurrency and audit attribution must be defined.
-Cross-tenant identifiers and unbounded queries must fail safely. Skills, agents and applications must use the tenant API or record service for business-state access.
-A platform owner must be able to keep only the agreed metadata in shared services.
-The shared control plane must hold identity and login, subscriptions, billing, and minimal routing and accounting metadata.
-Business records, detailed execution payloads, files, Cortex, code, applications and websites must remain in the isolated tenant environment.
-Data placement must be visible in architecture documentation and access tests. Multiple private containers or volumes may serve a tenant, but the database lifecycle must remain independent of an idle-paused code process.
-A GTM operator must be able to use one tenant-owned history for campaigns, leads and calling.
-Existing campaigns, campaign_calls, lead_queue and related lead, contact and calling data must migrate into typed tenant tables aligned with E13–E18.
-Identifiers, statuses, timestamps, consent, recordings and references, and outcomes must be preserved. The old shared path must be removed after verified cutover.
-A security owner must be able to prove tenant isolation across APIs, tools, workers, event consumers, scheduled jobs, logs, caches, volumes and network policies.
-Negative tests must prove that a tenant cannot address another tenant's records or files. Resource and storage limits must be enforced.
-An owner must be able to recover or leave with the complete business state.
-Export and restore must include the tenant database and artifact, source-document, Cortex and application manifests, together with permitted control metadata.
-Checksums, schema version, permissions and restoration evidence must be recorded, and restoration must not expose data to another tenant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E37" s="28" t="s">
+        <v>1272</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="27" t="s">
         <v>1077</v>
       </c>
@@ -17371,31 +17485,11 @@
       <c r="D38" s="26">
         <v>1</v>
       </c>
-      <c r="E38" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — tenant runtime, generated software and hosting
-Purpose: a tenant must be able to create and operate generated tools, internal applications and websites within its own isolated runtime. Depends on E01/E02/E03/E04/E08/E09/E12/E36, with generated-code promotion governed by E32. Tenant-local placement follows D25 and solution design follows D30. References: the tenant and ad hoc backlog and the operating model.
-A tenant must be able to run generated code and tools without gaining host access.
-Tenant containers must use versioned runtime images, isolated processes, network and credential policies, CPU, memory and time limits, and metering.
-Workers must never silently fall back to host filesystems or credentials.
-A capability owner must be able to reuse generated code safely.
-Source code, dependencies, tests, configuration references and build provenance must be stored in tenant-local versioned repositories.
-Workers must reload pinned versions. Changes must be reviewed, evaluated, promoted and rolled back through E32.
-An owner must be able to request an internal app for a business need.
-The request must become a tenant-local specification covering data tables and APIs, UI, workflows, permissions, limits and acceptance tests.
-The app must be previewable, editable and versioned before deployment.
-An administrator must be able to operate an app under the same platform controls as other work.
-App requests must use the tenant API and approved Skills or tools. Deployments must be isolated, observable, cancellable and auditable.
-Upgrades and rollback must preserve records and handle active-run behavior correctly.
-A tenant must be able to build, preview and host a website.
-Source, assets, builds, preview URL and publication state must be tenant-owned. Provider and domain configuration must be explicit and portable.
-Publication must require permissions, safety checks and a rollback capability.
-An operator must be able to find and manage source mirrors, uploads, artifacts, code, apps and site builds in stable tenant-storage folders.
-File metadata must include owner, provenance, version, retention and checksum. Quotas, alerts, deletion and restore must be enforced.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E38" s="28" t="s">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="27" t="s">
         <v>1105</v>
       </c>
@@ -17408,33 +17502,11 @@
       <c r="D39" s="26">
         <v>1</v>
       </c>
-      <c r="E39" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — Cortex knowledge graph and legacy RAG retirement
-Purpose: tenant agents must use traceable, editable knowledge and procedural memory built from original source material. The new Cortex path must replace the legacy document-ingestion and RAG implementation. Depends on E01/E02/E05/E06/E09/E10/E12/E36/E37. D27 defines acquisition and cutover, with D25 keeping the data tenant-local. References: the tenant and ad hoc backlog, product decisions and the source-coverage review.
-A new tenant must be able to teach the system about the company in a clear sequence.
-Registration must trigger bounded research of the company website, followed by requests for relevant uploads and connections to Google Drive, OneDrive, SharePoint and other approved sources.
-Pragya must show progress, consent, scope and failures.
-A tenant must be able to keep original files unchanged and mirror updates predictably.
-Originals must be saved in tenant folders with source URI, path, version, checksum, timestamps and synchronization cursor.
-Resynchronization, renaming, deletion and permission changes must be represented without silently overwriting provenance.
-An operator must be able to inspect and edit the tenant knowledge graph.
-Entities, relationships, procedures, assumptions and confidence must link to exact source documents and locations.
-Edits must retain version, author and reason. Retrieval must be tenant-scoped and permission-aware.
-An agent must be able to use Cortex evidence during work.
-Skills must receive citations, provenance, freshness and access decisions. Conflicting or missing evidence must be surfaced for review.
-Procedural updates must be testable before they affect approved workflows.
-A platform owner must be able to retire the legacy document-ingestion and RAG implementation completely.
-The migration must inventory old document and chunk tables, endpoints, jobs, indexes and flags, and move the required evidence into Cortex.
-After cutover, no production path may read or write the legacy store. Old code and tables must be removed, except for an explicitly isolated legal archive where required.
-Extraction and search must remain capabilities of the new Cortex path, with no parallel legacy RAG store or live dual-write path.
-An operator must be able to verify that cutover preserved the required knowledge.
-Replay and comparison must prove source coverage, links, permissions and retrieval behavior. Dashboards must identify orphaned originals and originals that have not been ingested.
-Rollback must be limited to versions of the new Cortex implementation and must not re-enable the retired RAG path.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E39" s="28" t="s">
+        <v>1274</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="27" t="s">
         <v>1133</v>
       </c>
@@ -17447,32 +17519,11 @@
       <c r="D40" s="26">
         <v>3</v>
       </c>
-      <c r="E40" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — Pragya solution design and ad hoc workbench
-Purpose: Pragya must be the single human workspace for packaged business operations and finite, one-off work, with every new solution designed collaboratively before deployment. Depends on E03/E05/E07/E08/E10/E12/E31/E33/E36/E38. D26 confirms voice-first operation with text and visual controls, D30 requires a shared solution blueprint and D32 confirms ad hoc work without mandatory pack activation. References: the tenant and ad hoc backlog, the operating model and product decisions.
-An owner must be able to describe a finite business goal outside a standard package.
-Pragya must accept the goal, constraints, source data and desired outputs and propose a bounded one-off plan.
-The task must not require a permanent agent hierarchy or activation of a Solo, MSME, startup or enterprise pack.
-An analyst must be able to turn raw data into a defensible financial model, market study or presentation.
-The run must select approved Skills, models and tools, record assumptions and calculations, cite evidence and produce editable artifacts.
-Material uncertainty and external effects must receive the required review.
-A tenant must be able to brainstorm a proposed solution with Pragya before deployment.
-A full solution-architect Meta Agent must turn the conversation into an editable blueprint covering goals, users, records, Skills and tools, integrations, events, schedules, permissions, budgets, risks, tests and success measures.
-Unresolved assumptions must remain visible.
-The tenant and Pragya must be able to edit the same design without losing decisions.
-Voice, text and visual controls must edit one versioned specification, with near-real-time presence and conflict handling.
-Changes must show authorship, differences, conflicts and approval state. Deployment must remain blocked until required reviewers approve the blueprint.
-A human operator must be able to access supported business functions through one workspace.
-Pragya must support voice-first and text interaction, contextual visual controls, generated analytics and drill-down.
-Every action must still use authorized platform APIs or Skills and retain audit history and provenance.
-An operator must be able to stop unsafe work immediately through a prominent, authenticated control.
-Stop must revoke eligible execution, prevent queued effects, settle known usage and show deterministic status.
-The stop control must work when voice, a model or a secondary channel is unavailable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25" ht="409.5" customHeight="1">
+      <c r="E40" s="28" t="s">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="27" t="s">
         <v>1161</v>
       </c>
@@ -17485,27 +17536,8 @@
       <c r="D41" s="26">
         <v>1</v>
       </c>
-      <c r="E41" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Functional requirements — optional Graph/Loop operating model and digital twin
-Purpose: tenants that need organizational modeling must be able to traverse and operate a Graph → Loop → Process → Agent → Skill → Action structure. Graph and Loop are optional, and ordinary workflows must remain valid without them. Depends on E03/E06/E07/E08/E10/E31/E33/E39. D07 defines the optional hierarchy and D31 defines the digital-twin experience, with E33's Design Gate preceding the new frontend. References: the tenant and ad hoc backlog and product decisions.
-An owner must be able to model the whole business as an optional Graph, with each Loop representing a department or function.
-Processes must retain their workflow meaning, Agents their role meaning, Skills their reusable-capability meaning, and Actions their tool-wrapper meaning.
-Every node must have a version, owner, policy, budget and data scope.
-An administrator must be able to validate and compile the hierarchy into executable work.
-References must resolve to versioned Skills and Actions. Permissions, budgets, memory scope, schedules and event subscriptions must be checked before activation.
-Cycles, duplicate ownership and unresolved nodes must fail with actionable diagnostics.
-An owner must be able to zoom from the business overview to an individual action through the new frontend's isometric digital twin.
-The view must traverse Graph, Loop, Process, Agent, Skill and Action where enabled and show dependencies and live status.
-The organizational Graph must be clearly distinguishable from a workflow dependency graph and the evidence-based knowledge graph. Available levels must be shown without forcing the optional hierarchy on every tenant.
-An operator must be able to edit the model visually and inspect its evidence.
-Visual editing must use the same versioned blueprint as Pragya, show the impact on permissions, budgets and runs, and link analytics to tenant records and source documents.
-An accessible alternative to the 3D view must be available.
-A business owner must be able to add or reorganize departments without duplicating execution.
-Adding or removing Loops must recompute routing, policy inheritance, budgets and reporting. Existing runs must retain their pinned versions, and event and schedule subscriptions must remain idempotent.
-A tenant without the hierarchy must still be able to run flat Process, Agent, Skill and Action workflows and ad hoc jobs with equivalent authorization, observability and stop controls.
-Enabling the hierarchy must be reversible and must not copy executable Skill versions or require extra model calls at every organizational level.</t>
-        </is>
+      <c r="E41" s="28" t="s">
+        <v>1276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>